<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 060526.xlsx 	modified:   public/data/meta.json 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1816" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6D1FD92-23DD-4E1F-9011-22BB8182711C}"/>
+  <xr:revisionPtr revIDLastSave="1818" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABC19F9B-1700-4375-B506-B4E03CACA1D9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1714,9 +1714,6 @@
     <t>Evaluation End Year</t>
   </si>
   <si>
-    <t>ACCSION is a large-scale CCS project at Aalborg Portland’s cement plant in Aalborg, Denmark, developed with Air Liquide to establish an integrated onshore carbon capture, transport, and storage chain. It captures CO₂ from both grey and white cement production using Cryocap™ technology and transports it by pipeline to onshore storage in Denmark. The project will capture about 1.4–1.42 MtCO₂ per year and avoid around 1.5 MtCO₂ annually, including benefits from surplus heat recovery. Around 80 MW of excess heat will be supplied to district heating. The project aims to enable near net-zero scope 1 emissions and demonstrate a scalable CCS model for heavy industry.</t>
-  </si>
-  <si>
     <t>Capture: Air Liquide Cryocap™ cryogenic CO₂ capture system, capturing CO₂ from flue-gas streams in a single integrated setup.
 Transport: Pipeline transport from the Aalborg cement site to a CO₂ reception/transport infrastructure.
 Storage: Onshore geological storage in Denmark / onshore CO₂ storage facilities (exact final storage formation/site not confirmed).
@@ -2490,6 +2487,9 @@
   </si>
   <si>
     <t>Cancelled</t>
+  </si>
+  <si>
+    <t>ACCSION is a large-scale CCS project at Aalborg Portland’s cement plant in Aalborg, Denmark, developed with Air Liquide to establish an integrated onshore carbon capture, transport, and storage chain. It captures CO₂ from both grey and white cement production using Cryocap™ technology and transports it by pipeline to onshore storage in Denmark. The project will capture about 1.4 MtCO₂ per year and avoid around 1.5 MtCO₂ annually, including benefits from surplus heat recovery. Around 80 MW of excess heat will be supplied to district heating. Aalborg portland recently won Danish CCS tender. The funding pool totals €3.85 billion and is central to Denmark’s strategy for cutting emissions, with Aalborg Portland now set to receive ongoing funding from it for each ton of captured and stored CO₂.</t>
   </si>
 </sst>
 </file>
@@ -4022,7 +4022,7 @@
         <v>74</v>
       </c>
       <c r="Q1" s="28" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="R1" s="28" t="s">
         <v>335</v>
@@ -4067,7 +4067,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" ht="148.19999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>87</v>
       </c>
@@ -4129,7 +4129,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V2" s="24">
         <v>57.062100000000001</v>
@@ -4144,22 +4144,22 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
       <c r="AB2" s="46" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AC2" s="30" t="s">
+        <v>593</v>
+      </c>
+      <c r="AD2" s="30" t="s">
         <v>336</v>
       </c>
-      <c r="AD2" s="30" t="s">
-        <v>337</v>
-      </c>
       <c r="AE2" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4167,7 +4167,7 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>242</v>
@@ -4224,7 +4224,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V3" s="24">
         <v>44.464755134852901</v>
@@ -4236,10 +4236,10 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4248,13 +4248,13 @@
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="AD3" s="30" t="s">
         <v>392</v>
       </c>
-      <c r="AD3" s="30" t="s">
-        <v>393</v>
-      </c>
       <c r="AE3" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4274,7 +4274,7 @@
         <v>52</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>288</v>
@@ -4319,7 +4319,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V4" s="26">
         <v>43.327720234653299</v>
@@ -4331,22 +4331,22 @@
         <v>95</v>
       </c>
       <c r="Y4" s="34" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Z4" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA4" s="34" t="s">
         <v>289</v>
       </c>
       <c r="AB4" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AC4" s="34" t="s">
+        <v>339</v>
+      </c>
+      <c r="AD4" s="34" t="s">
         <v>340</v>
-      </c>
-      <c r="AD4" s="34" t="s">
-        <v>341</v>
       </c>
       <c r="AE4" s="62" t="s">
         <v>27</v>
@@ -4357,13 +4357,13 @@
         <v>119</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4399,7 +4399,7 @@
         <v>92</v>
       </c>
       <c r="P5" s="32" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="Q5" s="32">
         <v>2030</v>
@@ -4414,7 +4414,7 @@
         <v>170000000</v>
       </c>
       <c r="U5" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V5" s="24">
         <v>46.809800000000003</v>
@@ -4429,22 +4429,22 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
       <c r="AB5" s="46" t="s">
+        <v>352</v>
+      </c>
+      <c r="AC5" s="30" t="s">
         <v>353</v>
       </c>
-      <c r="AC5" s="30" t="s">
+      <c r="AD5" s="30" t="s">
         <v>354</v>
       </c>
-      <c r="AD5" s="30" t="s">
-        <v>355</v>
-      </c>
       <c r="AE5" s="63" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="6" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4455,7 +4455,7 @@
         <v>278</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D6" s="30" t="s">
         <v>150</v>
@@ -4509,7 +4509,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V6" s="23" t="s">
         <v>92</v>
@@ -4524,22 +4524,22 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA6" s="30" t="s">
         <v>280</v>
       </c>
       <c r="AB6" s="46" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="7" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4604,7 +4604,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V7" s="24">
         <v>43.232830995956597</v>
@@ -4619,25 +4619,25 @@
         <v>334</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
       <c r="AB7" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="AC7" s="30" t="s">
+        <v>359</v>
+      </c>
+      <c r="AD7" s="30" t="s">
         <v>361</v>
       </c>
-      <c r="AC7" s="30" t="s">
-        <v>360</v>
-      </c>
-      <c r="AD7" s="30" t="s">
-        <v>362</v>
-      </c>
       <c r="AE7" s="63" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AF7" s="29" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -4687,7 +4687,7 @@
         <v>92</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="Q8" s="32">
         <v>2029</v>
@@ -4702,7 +4702,7 @@
         <v>115000000</v>
       </c>
       <c r="U8" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V8" s="24">
         <v>50.575420999999999</v>
@@ -4717,22 +4717,22 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AE8" s="63" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4743,19 +4743,19 @@
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4797,7 +4797,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V9" s="26">
         <v>37.960247145532399</v>
@@ -4809,25 +4809,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
       <c r="AE9" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4835,13 +4835,13 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
@@ -4907,19 +4907,19 @@
         <v>306</v>
       </c>
       <c r="Z10" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA10" s="30" t="s">
         <v>307</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4933,7 +4933,7 @@
         <v>266</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>150</v>
@@ -4942,10 +4942,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4987,7 +4987,7 @@
         <v>10206000</v>
       </c>
       <c r="U11" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V11" s="24">
         <v>59.592303479664103</v>
@@ -4999,25 +4999,25 @@
         <v>244</v>
       </c>
       <c r="Y11" s="30" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="Z11" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA11" s="30" t="s">
         <v>267</v>
       </c>
       <c r="AB11" s="46" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AC11" s="30" t="s">
+        <v>419</v>
+      </c>
+      <c r="AD11" s="30" t="s">
         <v>420</v>
       </c>
-      <c r="AD11" s="30" t="s">
-        <v>421</v>
-      </c>
       <c r="AE11" s="63" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5097,22 +5097,22 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
       <c r="AB12" s="46" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="AC12" s="34" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AE12" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="13" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5189,10 +5189,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5201,13 +5201,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
+        <v>380</v>
+      </c>
+      <c r="AD13" s="34" t="s">
         <v>381</v>
       </c>
-      <c r="AD13" s="34" t="s">
-        <v>382</v>
-      </c>
       <c r="AE13" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="14" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5218,7 +5218,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5272,7 +5272,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V14" s="26">
         <v>44.826999999999998</v>
@@ -5287,22 +5287,22 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AC14" s="34" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD14" s="34" t="s">
         <v>409</v>
       </c>
-      <c r="AD14" s="34" t="s">
-        <v>410</v>
-      </c>
       <c r="AE14" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="15" spans="1:32" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5367,7 +5367,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V15" s="26">
         <v>43.186100000000003</v>
@@ -5382,20 +5382,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="16" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5418,7 +5418,7 @@
         <v>275</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5460,7 +5460,7 @@
         <v>146415990</v>
       </c>
       <c r="U16" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V16" s="24">
         <v>45.290985428950698</v>
@@ -5472,25 +5472,25 @@
         <v>244</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA16" s="30" t="s">
         <v>286</v>
       </c>
       <c r="AB16" s="46" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AC16" s="30" t="s">
+        <v>425</v>
+      </c>
+      <c r="AD16" s="30" t="s">
         <v>426</v>
       </c>
-      <c r="AD16" s="30" t="s">
-        <v>427</v>
-      </c>
       <c r="AE16" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5513,7 +5513,7 @@
         <v>253</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5555,7 +5555,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V17" s="23">
         <v>51.870851200822599</v>
@@ -5567,10 +5567,10 @@
         <v>244</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA17" s="30" t="s">
         <v>254</v>
@@ -5579,10 +5579,10 @@
         <v>255</v>
       </c>
       <c r="AC17" s="30" t="s">
+        <v>429</v>
+      </c>
+      <c r="AD17" s="30" t="s">
         <v>430</v>
-      </c>
-      <c r="AD17" s="30" t="s">
-        <v>431</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5650,7 +5650,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V18" s="24">
         <v>52.489100000000001</v>
@@ -5665,7 +5665,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5674,13 +5674,13 @@
         <v>208</v>
       </c>
       <c r="AC18" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="AD18" s="30" t="s">
         <v>386</v>
       </c>
-      <c r="AD18" s="30" t="s">
-        <v>387</v>
-      </c>
       <c r="AE18" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5745,7 +5745,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V19" s="26">
         <v>50.569000000000003</v>
@@ -5760,13 +5760,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5786,10 +5786,10 @@
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5798,7 +5798,7 @@
         <v>235</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5855,7 +5855,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5864,13 +5864,13 @@
         <v>240</v>
       </c>
       <c r="AC20" s="34" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD20" s="34" t="s">
         <v>434</v>
       </c>
-      <c r="AD20" s="34" t="s">
-        <v>435</v>
-      </c>
       <c r="AE20" s="66" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5881,10 +5881,10 @@
         <v>302</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5923,10 +5923,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="36" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="R21" s="36" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="S21" s="22" t="s">
         <v>122</v>
@@ -5935,7 +5935,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V21" s="26">
         <v>41.352637812781921</v>
@@ -5947,25 +5947,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="Z21" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA21" s="34" t="s">
         <v>303</v>
       </c>
       <c r="AB21" s="46" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="AC21" s="34" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AD21" s="34" t="s">
         <v>304</v>
       </c>
       <c r="AE21" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6042,25 +6042,25 @@
         <v>244</v>
       </c>
       <c r="Y22" s="29" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
       <c r="AB22" s="46" t="s">
+        <v>438</v>
+      </c>
+      <c r="AC22" s="30" t="s">
         <v>439</v>
       </c>
-      <c r="AC22" s="30" t="s">
+      <c r="AD22" s="30" t="s">
         <v>440</v>
       </c>
-      <c r="AD22" s="30" t="s">
-        <v>441</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6080,10 +6080,10 @@
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6137,25 +6137,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>443</v>
+      </c>
+      <c r="AC23" s="34" t="s">
         <v>444</v>
       </c>
-      <c r="AC23" s="34" t="s">
+      <c r="AD23" s="34" t="s">
         <v>445</v>
       </c>
-      <c r="AD23" s="34" t="s">
-        <v>446</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6166,7 +6166,7 @@
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>150</v>
@@ -6175,10 +6175,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
+        <v>452</v>
+      </c>
+      <c r="G24" s="72" t="s">
         <v>453</v>
-      </c>
-      <c r="G24" s="72" t="s">
-        <v>454</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6232,25 +6232,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AC24" s="34" t="s">
+        <v>454</v>
+      </c>
+      <c r="AD24" s="34" t="s">
         <v>455</v>
       </c>
-      <c r="AD24" s="34" t="s">
-        <v>456</v>
-      </c>
       <c r="AE24" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6270,10 +6270,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6315,7 +6315,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V25" s="26">
         <v>45.515127894849797</v>
@@ -6327,25 +6327,25 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
+        <v>588</v>
+      </c>
+      <c r="Z25" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="AA25" s="34" t="s">
         <v>589</v>
       </c>
-      <c r="Z25" s="34" t="s">
-        <v>580</v>
-      </c>
-      <c r="AA25" s="34" t="s">
-        <v>590</v>
-      </c>
       <c r="AB25" s="46" t="s">
+        <v>448</v>
+      </c>
+      <c r="AC25" s="34" t="s">
         <v>449</v>
       </c>
-      <c r="AC25" s="34" t="s">
+      <c r="AD25" s="34" t="s">
         <v>450</v>
       </c>
-      <c r="AD25" s="34" t="s">
-        <v>451</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6356,7 +6356,7 @@
         <v>258</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6410,7 +6410,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V26" s="22">
         <v>59.121267699503399</v>
@@ -6422,10 +6422,10 @@
         <v>244</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA26" s="34" t="s">
         <v>260</v>
@@ -6434,13 +6434,13 @@
         <v>261</v>
       </c>
       <c r="AC26" s="34" t="s">
+        <v>584</v>
+      </c>
+      <c r="AD26" s="34" t="s">
         <v>585</v>
       </c>
-      <c r="AD26" s="34" t="s">
-        <v>586</v>
-      </c>
       <c r="AE26" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6463,7 +6463,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6517,10 +6517,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6529,13 +6529,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
+        <v>459</v>
+      </c>
+      <c r="AD27" s="30" t="s">
         <v>460</v>
       </c>
-      <c r="AD27" s="30" t="s">
-        <v>461</v>
-      </c>
       <c r="AE27" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6549,7 +6549,7 @@
         <v>225</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6612,25 +6612,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>463</v>
+      </c>
+      <c r="AC28" s="30" t="s">
         <v>464</v>
       </c>
-      <c r="AC28" s="30" t="s">
+      <c r="AD28" s="30" t="s">
         <v>465</v>
       </c>
-      <c r="AD28" s="30" t="s">
-        <v>466</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6695,7 +6695,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V29" s="24">
         <v>51.297800000000002</v>
@@ -6707,10 +6707,10 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6719,13 +6719,13 @@
         <v>199</v>
       </c>
       <c r="AC29" s="30" t="s">
+        <v>467</v>
+      </c>
+      <c r="AD29" s="30" t="s">
         <v>468</v>
       </c>
-      <c r="AD29" s="30" t="s">
-        <v>469</v>
-      </c>
       <c r="AE29" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6733,19 +6733,19 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>312</v>
@@ -6790,7 +6790,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V30" s="22">
         <v>60.618241659279597</v>
@@ -6802,25 +6802,25 @@
         <v>244</v>
       </c>
       <c r="Y30" s="34" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA30" s="34" t="s">
         <v>313</v>
       </c>
       <c r="AB30" s="47" t="s">
+        <v>494</v>
+      </c>
+      <c r="AC30" s="34" t="s">
         <v>495</v>
       </c>
-      <c r="AC30" s="34" t="s">
+      <c r="AD30" s="34" t="s">
         <v>496</v>
       </c>
-      <c r="AD30" s="34" t="s">
-        <v>497</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6885,7 +6885,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V31" s="26">
         <v>51.618000000000002</v>
@@ -6900,7 +6900,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -6909,13 +6909,13 @@
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
+        <v>406</v>
+      </c>
+      <c r="AD31" s="34" t="s">
         <v>407</v>
       </c>
-      <c r="AD31" s="34" t="s">
-        <v>408</v>
-      </c>
       <c r="AE31" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6935,10 +6935,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6992,25 +6992,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="Z32" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA32" s="34" t="s">
         <v>276</v>
       </c>
       <c r="AB32" s="46" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="AC32" s="34" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AD32" s="34" t="s">
         <v>277</v>
       </c>
       <c r="AE32" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7090,22 +7090,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="AC33" s="30" t="s">
+        <v>471</v>
+      </c>
+      <c r="AD33" s="30" t="s">
         <v>472</v>
       </c>
-      <c r="AD33" s="30" t="s">
-        <v>473</v>
-      </c>
       <c r="AE33" s="66" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7119,7 +7119,7 @@
         <v>225</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
@@ -7168,7 +7168,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V34" s="23">
         <v>43.151000000000003</v>
@@ -7180,10 +7180,10 @@
         <v>244</v>
       </c>
       <c r="Y34" s="30" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="Z34" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA34" s="30" t="s">
         <v>292</v>
@@ -7192,13 +7192,13 @@
         <v>293</v>
       </c>
       <c r="AC34" s="30" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD34" s="30" t="s">
         <v>476</v>
       </c>
-      <c r="AD34" s="30" t="s">
-        <v>477</v>
-      </c>
       <c r="AE34" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7209,10 +7209,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7221,7 +7221,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7278,19 +7278,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AC35" s="34" t="s">
+        <v>371</v>
+      </c>
+      <c r="AD35" s="34" t="s">
         <v>372</v>
-      </c>
-      <c r="AD35" s="34" t="s">
-        <v>373</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7304,7 +7304,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7358,7 +7358,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V36" s="26">
         <v>51.1339349</v>
@@ -7370,25 +7370,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="AC36" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="AD36" s="34" t="s">
         <v>480</v>
       </c>
-      <c r="AD36" s="34" t="s">
-        <v>481</v>
-      </c>
       <c r="AE36" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7399,10 +7399,10 @@
         <v>281</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
@@ -7453,7 +7453,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V37" s="26">
         <v>50.529000000000003</v>
@@ -7468,22 +7468,22 @@
         <v>284</v>
       </c>
       <c r="Z37" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA37" s="34" t="s">
         <v>285</v>
       </c>
       <c r="AB37" s="46" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AC37" s="34" t="s">
+        <v>481</v>
+      </c>
+      <c r="AD37" s="34" t="s">
         <v>482</v>
       </c>
-      <c r="AD37" s="34" t="s">
-        <v>483</v>
-      </c>
       <c r="AE37" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7548,7 +7548,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V38" s="26">
         <v>38.129899999999999</v>
@@ -7560,25 +7560,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
       <c r="AB38" s="46" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AC38" s="34" t="s">
+        <v>402</v>
+      </c>
+      <c r="AD38" s="34" t="s">
         <v>403</v>
       </c>
-      <c r="AD38" s="34" t="s">
-        <v>404</v>
-      </c>
       <c r="AE38" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7589,7 +7589,7 @@
         <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7653,25 +7653,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA39" s="30" t="s">
         <v>311</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7685,7 +7685,7 @@
         <v>219</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -7736,7 +7736,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V40" s="24">
         <v>37.916800000000002</v>
@@ -7751,7 +7751,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7760,13 +7760,13 @@
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
+        <v>486</v>
+      </c>
+      <c r="AD40" s="30" t="s">
         <v>487</v>
       </c>
-      <c r="AD40" s="30" t="s">
-        <v>488</v>
-      </c>
       <c r="AE40" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7846,22 +7846,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="AC41" s="30" t="s">
+        <v>488</v>
+      </c>
+      <c r="AD41" s="30" t="s">
         <v>489</v>
       </c>
-      <c r="AD41" s="30" t="s">
-        <v>490</v>
-      </c>
       <c r="AE41" s="66" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7926,7 +7926,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V42" s="26">
         <v>44.968299999999999</v>
@@ -7941,22 +7941,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7964,13 +7964,13 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
+        <v>374</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>376</v>
-      </c>
       <c r="D43" s="30" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
@@ -8021,7 +8021,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V43" s="26">
         <v>51.976999999999997</v>
@@ -8036,22 +8036,22 @@
         <v>257</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>376</v>
+      </c>
+      <c r="AC43" s="34" t="s">
         <v>377</v>
       </c>
-      <c r="AC43" s="34" t="s">
+      <c r="AD43" s="34" t="s">
         <v>378</v>
       </c>
-      <c r="AD43" s="34" t="s">
-        <v>379</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8116,7 +8116,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V44" s="26">
         <v>50.406342306737002</v>
@@ -8128,25 +8128,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>498</v>
+      </c>
+      <c r="AC44" s="34" t="s">
         <v>499</v>
       </c>
-      <c r="AC44" s="34" t="s">
+      <c r="AD44" s="34" t="s">
         <v>500</v>
       </c>
-      <c r="AD44" s="34" t="s">
-        <v>501</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8157,16 +8157,16 @@
         <v>264</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8211,7 +8211,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V45" s="22">
         <v>59.2181</v>
@@ -8223,7 +8223,7 @@
         <v>244</v>
       </c>
       <c r="Y45" s="34" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="Z45" s="34" t="s">
         <v>225</v>
@@ -8232,16 +8232,16 @@
         <v>265</v>
       </c>
       <c r="AB45" s="46" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="AC45" s="34" t="s">
+        <v>504</v>
+      </c>
+      <c r="AD45" s="34" t="s">
         <v>505</v>
       </c>
-      <c r="AD45" s="34" t="s">
-        <v>506</v>
-      </c>
       <c r="AE45" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8321,22 +8321,22 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
       <c r="AB46" s="46" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="AC46" s="30" t="s">
+        <v>399</v>
+      </c>
+      <c r="AD46" s="30" t="s">
         <v>400</v>
       </c>
-      <c r="AD46" s="30" t="s">
-        <v>401</v>
-      </c>
       <c r="AE46" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8347,7 +8347,7 @@
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>150</v>
@@ -8356,10 +8356,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>507</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>508</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8416,22 +8416,22 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AC47" s="30" t="s">
+        <v>508</v>
+      </c>
+      <c r="AD47" s="30" t="s">
         <v>509</v>
       </c>
-      <c r="AD47" s="30" t="s">
-        <v>510</v>
-      </c>
       <c r="AE47" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8439,7 +8439,7 @@
         <v>87</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
@@ -8451,10 +8451,10 @@
         <v>58</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8496,7 +8496,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="V48" s="22">
         <v>58.099057767351503</v>
@@ -8508,25 +8508,25 @@
         <v>244</v>
       </c>
       <c r="Y48" s="34" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA48" s="34" t="s">
         <v>308</v>
       </c>
       <c r="AB48" s="47" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AD48" s="34" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8546,10 +8546,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8591,7 +8591,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V49" s="26">
         <v>56.787056035485499</v>
@@ -8606,22 +8606,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>514</v>
+      </c>
+      <c r="AC49" s="34" t="s">
         <v>515</v>
       </c>
-      <c r="AC49" s="34" t="s">
+      <c r="AD49" s="34" t="s">
         <v>516</v>
       </c>
-      <c r="AD49" s="34" t="s">
-        <v>517</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8635,7 +8635,7 @@
         <v>225</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
@@ -8674,7 +8674,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V50" s="26">
         <v>48.096166502584701</v>
@@ -8686,7 +8686,7 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="Z50" s="34" t="s">
         <v>225</v>
@@ -8695,16 +8695,16 @@
         <v>211</v>
       </c>
       <c r="AB50" s="46" t="s">
+        <v>518</v>
+      </c>
+      <c r="AC50" s="34" t="s">
         <v>519</v>
       </c>
-      <c r="AC50" s="34" t="s">
+      <c r="AD50" s="34" t="s">
         <v>520</v>
       </c>
-      <c r="AD50" s="34" t="s">
-        <v>521</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8724,10 +8724,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8781,25 +8781,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>522</v>
+      </c>
+      <c r="AC51" s="30" t="s">
         <v>523</v>
       </c>
-      <c r="AC51" s="30" t="s">
+      <c r="AD51" s="30" t="s">
         <v>524</v>
       </c>
-      <c r="AD51" s="30" t="s">
-        <v>525</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8864,7 +8864,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V52" s="26">
         <v>60.306100000000001</v>
@@ -8879,7 +8879,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8894,7 +8894,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8905,7 +8905,7 @@
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8917,7 +8917,7 @@
         <v>235</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8959,7 +8959,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V53" s="24">
         <v>64.037112316635401</v>
@@ -8971,22 +8971,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
       <c r="AB53" s="46" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AC53" s="30" t="s">
+        <v>531</v>
+      </c>
+      <c r="AD53" s="30" t="s">
         <v>532</v>
-      </c>
-      <c r="AD53" s="30" t="s">
-        <v>533</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -9000,19 +9000,19 @@
         <v>272</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="G54" s="30" t="s">
         <v>534</v>
-      </c>
-      <c r="G54" s="30" t="s">
-        <v>535</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9054,7 +9054,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V54" s="24">
         <v>59.127044152710397</v>
@@ -9066,25 +9066,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA54" s="30" t="s">
         <v>273</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>535</v>
+      </c>
+      <c r="AC54" s="30" t="s">
         <v>536</v>
       </c>
-      <c r="AC54" s="30" t="s">
+      <c r="AD54" s="30" t="s">
         <v>537</v>
       </c>
-      <c r="AD54" s="30" t="s">
-        <v>538</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9095,19 +9095,19 @@
         <v>262</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9149,7 +9149,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V55" s="23">
         <v>57.788622470324199</v>
@@ -9161,23 +9161,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
         <v>263</v>
       </c>
       <c r="AC55" s="30" t="s">
+        <v>383</v>
+      </c>
+      <c r="AD55" s="30" t="s">
         <v>384</v>
       </c>
-      <c r="AD55" s="30" t="s">
-        <v>385</v>
-      </c>
       <c r="AE55" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9197,10 +9197,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>542</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>543</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9254,25 +9254,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>544</v>
+      </c>
+      <c r="AC56" s="30" t="s">
         <v>545</v>
       </c>
-      <c r="AC56" s="30" t="s">
+      <c r="AD56" s="30" t="s">
         <v>546</v>
       </c>
-      <c r="AD56" s="30" t="s">
-        <v>547</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9283,19 +9283,19 @@
         <v>299</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9337,7 +9337,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="33" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V57" s="24">
         <v>40.8482802817337</v>
@@ -9349,10 +9349,10 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="Z57" s="30" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AA57" s="30" t="s">
         <v>300</v>
@@ -9361,13 +9361,13 @@
         <v>301</v>
       </c>
       <c r="AC57" s="30" t="s">
+        <v>549</v>
+      </c>
+      <c r="AD57" s="30" t="s">
         <v>550</v>
       </c>
-      <c r="AD57" s="30" t="s">
-        <v>551</v>
-      </c>
       <c r="AE57" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9381,7 +9381,7 @@
         <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9444,7 +9444,7 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="Z58" s="30" t="s">
         <v>225</v>
@@ -9453,16 +9453,16 @@
         <v>230</v>
       </c>
       <c r="AB58" s="46" t="s">
+        <v>558</v>
+      </c>
+      <c r="AC58" s="30" t="s">
         <v>559</v>
       </c>
-      <c r="AC58" s="30" t="s">
+      <c r="AD58" s="30" t="s">
         <v>560</v>
       </c>
-      <c r="AD58" s="30" t="s">
-        <v>561</v>
-      </c>
       <c r="AE58" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9473,7 +9473,7 @@
         <v>294</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>150</v>
@@ -9539,10 +9539,10 @@
         <v>244</v>
       </c>
       <c r="Y59" s="34" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="Z59" s="34" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA59" s="34" t="s">
         <v>296</v>
@@ -9551,13 +9551,13 @@
         <v>297</v>
       </c>
       <c r="AC59" s="34" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="AD59" s="34" t="s">
         <v>298</v>
       </c>
       <c r="AE59" s="61" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9637,22 +9637,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
+        <v>553</v>
+      </c>
+      <c r="AC60" s="34" t="s">
         <v>554</v>
-      </c>
-      <c r="AC60" s="34" t="s">
-        <v>555</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9666,7 +9666,7 @@
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
@@ -9717,7 +9717,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="37" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="V61" s="26">
         <v>60.45333865137971</v>
@@ -9729,7 +9729,7 @@
         <v>244</v>
       </c>
       <c r="Y61" s="34" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="Z61" s="34" t="s">
         <v>225</v>
@@ -9738,16 +9738,16 @@
         <v>270</v>
       </c>
       <c r="AB61" s="46" t="s">
+        <v>556</v>
+      </c>
+      <c r="AC61" s="34" t="s">
         <v>557</v>
-      </c>
-      <c r="AC61" s="34" t="s">
-        <v>558</v>
       </c>
       <c r="AD61" s="34" t="s">
         <v>271</v>
       </c>
       <c r="AE61" s="65" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 060526.xlsx 	modified:   src/components/Legend.jsx 	modified:   src/components/Legend.module.css
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1818" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABC19F9B-1700-4375-B506-B4E03CACA1D9}"/>
+  <xr:revisionPtr revIDLastSave="1822" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BE9FB7F-7FA0-4A3F-A66D-587EBE2DAC86}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3074,36 +3074,27 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3125,6 +3116,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3446,40 +3446,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3496,12 +3496,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3510,12 +3510,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="74"/>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="74"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3524,12 +3524,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3538,12 +3538,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="76"/>
+      <c r="H9" s="76"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3552,12 +3552,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="74"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="74"/>
+      <c r="C10" s="76"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
+      <c r="F10" s="76"/>
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3566,12 +3566,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3580,24 +3580,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="74"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="74"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="74"/>
+      <c r="B15" s="76"/>
+      <c r="C15" s="76"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3609,11 +3609,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="77"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="75"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3622,14 +3622,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="75" t="s">
+      <c r="C17" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="76"/>
-      <c r="E17" s="76"/>
-      <c r="F17" s="76"/>
-      <c r="G17" s="76"/>
-      <c r="H17" s="77"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="75"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3638,14 +3638,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="79" t="s">
+      <c r="C18" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="77"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="74"/>
+      <c r="H18" s="75"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3654,14 +3654,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="77"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="75"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3670,14 +3670,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="79" t="s">
+      <c r="C20" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="76"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="77"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="75"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3686,14 +3686,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="75"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3702,14 +3702,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="79" t="s">
+      <c r="C22" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="77"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="74"/>
+      <c r="F22" s="74"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="75"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3718,14 +3718,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="75" t="s">
+      <c r="C23" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="77"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="75"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3734,14 +3734,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="79" t="s">
+      <c r="C24" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="77"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="75"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3750,26 +3750,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="75" t="s">
+      <c r="C25" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="77"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="75"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="73" t="s">
+      <c r="A28" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="74"/>
-      <c r="C28" s="74"/>
-      <c r="D28" s="74"/>
-      <c r="E28" s="74"/>
-      <c r="F28" s="74"/>
-      <c r="G28" s="74"/>
-      <c r="H28" s="74"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="76"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
+      <c r="H28" s="76"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3913,12 +3913,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3935,6 +3929,12 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9835,141 +9835,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="84" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="78" t="s">
         <v>315</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="93" t="s">
+      <c r="A4" s="90" t="s">
         <v>316</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="82" t="s">
+      <c r="B4" s="75"/>
+      <c r="C4" s="83" t="s">
         <v>317</v>
       </c>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="82" t="s">
+      <c r="B5" s="75"/>
+      <c r="C5" s="83" t="s">
         <v>318</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="88" t="s">
+      <c r="A6" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="82" t="s">
+      <c r="B6" s="75"/>
+      <c r="C6" s="83" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="77"/>
-      <c r="C7" s="82" t="s">
+      <c r="B7" s="75"/>
+      <c r="C7" s="83" t="s">
         <v>320</v>
       </c>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="92" t="s">
+      <c r="A8" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="77"/>
-      <c r="C8" s="82" t="s">
+      <c r="B8" s="75"/>
+      <c r="C8" s="83" t="s">
         <v>321</v>
       </c>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="85" t="s">
+      <c r="A9" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="77"/>
-      <c r="C9" s="82" t="s">
+      <c r="B9" s="75"/>
+      <c r="C9" s="83" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="77"/>
-      <c r="C10" s="82" t="s">
+      <c r="B10" s="75"/>
+      <c r="C10" s="83" t="s">
         <v>323</v>
       </c>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="73" t="s">
+      <c r="A12" s="78" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="74"/>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="84" t="s">
+      <c r="A13" s="92" t="s">
         <v>325</v>
       </c>
-      <c r="B13" s="77"/>
-      <c r="C13" s="82" t="s">
+      <c r="B13" s="75"/>
+      <c r="C13" s="83" t="s">
         <v>326</v>
       </c>
-      <c r="D13" s="74"/>
-      <c r="E13" s="74"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="91" t="s">
+      <c r="A14" s="88" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="77"/>
-      <c r="C14" s="82" t="s">
+      <c r="B14" s="75"/>
+      <c r="C14" s="83" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="74"/>
-      <c r="E14" s="74"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="76"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="86" t="s">
+      <c r="A15" s="82" t="s">
         <v>329</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="82" t="s">
+      <c r="B15" s="75"/>
+      <c r="C15" s="83" t="s">
         <v>330</v>
       </c>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
@@ -9984,6 +9984,13 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10000,13 +10007,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10014,26 +10014,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -10274,10 +10254,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10300,20 +10311,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 060526.xlsx 	modified:   public/data/meta.json 	modified:   public/data/projects.json 	modified:   src/components/FilterPanel.jsx 	modified:   src/components/Legend.jsx 	modified:   src/constants.js
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmeurope-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1822" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BE9FB7F-7FA0-4A3F-A66D-587EBE2DAC86}"/>
+  <xr:revisionPtr revIDLastSave="1824" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49E2393-40B6-402C-A971-F8F37DFD2767}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1714,12 +1714,6 @@
     <t>Evaluation End Year</t>
   </si>
   <si>
-    <t>Capture: Air Liquide Cryocap™ cryogenic CO₂ capture system, capturing CO₂ from flue-gas streams in a single integrated setup.
-Transport: Pipeline transport from the Aalborg cement site to a CO₂ reception/transport infrastructure.
-Storage: Onshore geological storage in Denmark / onshore CO₂ storage facilities (exact final storage formation/site not confirmed).
-Integration notes: renewable electricity supply for the capture plant, certified biogas use in kilns, digital monitoring, and recovery of ~80 MW surplus heat for district heating.</t>
-  </si>
-  <si>
     <t>BISCAY ECO AGGREGATES, S.L.</t>
   </si>
   <si>
@@ -2490,6 +2484,9 @@
   </si>
   <si>
     <t>ACCSION is a large-scale CCS project at Aalborg Portland’s cement plant in Aalborg, Denmark, developed with Air Liquide to establish an integrated onshore carbon capture, transport, and storage chain. It captures CO₂ from both grey and white cement production using Cryocap™ technology and transports it by pipeline to onshore storage in Denmark. The project will capture about 1.4 MtCO₂ per year and avoid around 1.5 MtCO₂ annually, including benefits from surplus heat recovery. Around 80 MW of excess heat will be supplied to district heating. Aalborg portland recently won Danish CCS tender. The funding pool totals €3.85 billion and is central to Denmark’s strategy for cutting emissions, with Aalborg Portland now set to receive ongoing funding from it for each ton of captured and stored CO₂.</t>
+  </si>
+  <si>
+    <t>The project uses the Air Liquide Cryocap™ cryogenic CO₂ capture system to capture CO₂ directly from flue-gas streams within a single integrated setup. The captured CO₂ is transported via pipeline from the Aalborg cement plant to a CO₂ transport infrastructure, before being sent to onshore geological storage facilities in Denmark. However, the exact final storage site has not yet been confirmed. The system is further supported by renewable electricity for the capture plant, certified biogas in the kilns, digital monitoring systems, and the recovery of approximately 80 MW of surplus heat for district heating applications.</t>
   </si>
 </sst>
 </file>
@@ -3074,27 +3071,36 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3118,15 +3124,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3143,6 +3140,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3446,40 +3447,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="78" t="s">
+      <c r="A4" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3496,12 +3497,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3510,12 +3511,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3524,12 +3525,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="76"/>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="76"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3538,12 +3539,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3552,12 +3553,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3566,12 +3567,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3580,24 +3581,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="78" t="s">
+      <c r="A15" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3609,11 +3610,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="75"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3622,14 +3623,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="74"/>
-      <c r="G17" s="74"/>
-      <c r="H17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="77"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3638,14 +3639,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="77" t="s">
+      <c r="C18" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="74"/>
-      <c r="H18" s="75"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3654,14 +3655,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="73" t="s">
+      <c r="C19" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="75"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3670,14 +3671,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="77" t="s">
+      <c r="C20" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="74"/>
-      <c r="H20" s="75"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="77"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3686,14 +3687,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="75"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3702,14 +3703,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="77" t="s">
+      <c r="C22" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="75"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3718,14 +3719,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="73" t="s">
+      <c r="C23" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="75"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="77"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3734,14 +3735,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="77" t="s">
+      <c r="C24" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
-      <c r="H24" s="75"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3750,26 +3751,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="73" t="s">
+      <c r="C25" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="74"/>
-      <c r="E25" s="74"/>
-      <c r="F25" s="74"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="75"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="78" t="s">
+      <c r="A28" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="76"/>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-      <c r="H28" s="76"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="74"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3913,6 +3914,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3929,12 +3936,6 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4022,7 +4023,7 @@
         <v>74</v>
       </c>
       <c r="Q1" s="28" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="R1" s="28" t="s">
         <v>335</v>
@@ -4129,7 +4130,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V2" s="24">
         <v>57.062100000000001</v>
@@ -4144,22 +4145,22 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
       <c r="AB2" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AC2" s="30" t="s">
+        <v>592</v>
+      </c>
+      <c r="AD2" s="30" t="s">
         <v>593</v>
       </c>
-      <c r="AD2" s="30" t="s">
-        <v>336</v>
-      </c>
       <c r="AE2" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4167,7 +4168,7 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>242</v>
@@ -4224,7 +4225,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V3" s="24">
         <v>44.464755134852901</v>
@@ -4236,10 +4237,10 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4248,13 +4249,13 @@
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
+        <v>390</v>
+      </c>
+      <c r="AD3" s="30" t="s">
         <v>391</v>
       </c>
-      <c r="AD3" s="30" t="s">
-        <v>392</v>
-      </c>
       <c r="AE3" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4274,7 +4275,7 @@
         <v>52</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>288</v>
@@ -4319,7 +4320,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V4" s="26">
         <v>43.327720234653299</v>
@@ -4331,22 +4332,22 @@
         <v>95</v>
       </c>
       <c r="Y4" s="34" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="Z4" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA4" s="34" t="s">
         <v>289</v>
       </c>
       <c r="AB4" s="46" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AC4" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="AD4" s="34" t="s">
         <v>339</v>
-      </c>
-      <c r="AD4" s="34" t="s">
-        <v>340</v>
       </c>
       <c r="AE4" s="62" t="s">
         <v>27</v>
@@ -4357,13 +4358,13 @@
         <v>119</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4399,7 +4400,7 @@
         <v>92</v>
       </c>
       <c r="P5" s="32" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q5" s="32">
         <v>2030</v>
@@ -4414,7 +4415,7 @@
         <v>170000000</v>
       </c>
       <c r="U5" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V5" s="24">
         <v>46.809800000000003</v>
@@ -4429,22 +4430,22 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
       <c r="AB5" s="46" t="s">
+        <v>351</v>
+      </c>
+      <c r="AC5" s="30" t="s">
         <v>352</v>
       </c>
-      <c r="AC5" s="30" t="s">
+      <c r="AD5" s="30" t="s">
         <v>353</v>
       </c>
-      <c r="AD5" s="30" t="s">
-        <v>354</v>
-      </c>
       <c r="AE5" s="63" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="6" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4455,7 +4456,7 @@
         <v>278</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D6" s="30" t="s">
         <v>150</v>
@@ -4509,7 +4510,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V6" s="23" t="s">
         <v>92</v>
@@ -4524,22 +4525,22 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA6" s="30" t="s">
         <v>280</v>
       </c>
       <c r="AB6" s="46" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4604,7 +4605,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V7" s="24">
         <v>43.232830995956597</v>
@@ -4619,25 +4620,25 @@
         <v>334</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
       <c r="AB7" s="46" t="s">
+        <v>359</v>
+      </c>
+      <c r="AC7" s="30" t="s">
+        <v>358</v>
+      </c>
+      <c r="AD7" s="30" t="s">
         <v>360</v>
       </c>
-      <c r="AC7" s="30" t="s">
-        <v>359</v>
-      </c>
-      <c r="AD7" s="30" t="s">
-        <v>361</v>
-      </c>
       <c r="AE7" s="63" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="AF7" s="29" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -4687,7 +4688,7 @@
         <v>92</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Q8" s="32">
         <v>2029</v>
@@ -4702,7 +4703,7 @@
         <v>115000000</v>
       </c>
       <c r="U8" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V8" s="24">
         <v>50.575420999999999</v>
@@ -4717,22 +4718,22 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AE8" s="63" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4743,19 +4744,19 @@
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4797,7 +4798,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V9" s="26">
         <v>37.960247145532399</v>
@@ -4809,25 +4810,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
       <c r="AE9" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4835,13 +4836,13 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
@@ -4907,19 +4908,19 @@
         <v>306</v>
       </c>
       <c r="Z10" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA10" s="30" t="s">
         <v>307</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4933,7 +4934,7 @@
         <v>266</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>150</v>
@@ -4942,10 +4943,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4987,7 +4988,7 @@
         <v>10206000</v>
       </c>
       <c r="U11" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V11" s="24">
         <v>59.592303479664103</v>
@@ -4999,25 +5000,25 @@
         <v>244</v>
       </c>
       <c r="Y11" s="30" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="Z11" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA11" s="30" t="s">
         <v>267</v>
       </c>
       <c r="AB11" s="46" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AC11" s="30" t="s">
+        <v>418</v>
+      </c>
+      <c r="AD11" s="30" t="s">
         <v>419</v>
       </c>
-      <c r="AD11" s="30" t="s">
-        <v>420</v>
-      </c>
       <c r="AE11" s="63" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5097,22 +5098,22 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
       <c r="AB12" s="46" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC12" s="34" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AE12" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="13" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5189,10 +5190,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5201,13 +5202,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
+        <v>379</v>
+      </c>
+      <c r="AD13" s="34" t="s">
         <v>380</v>
       </c>
-      <c r="AD13" s="34" t="s">
-        <v>381</v>
-      </c>
       <c r="AE13" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5218,7 +5219,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5272,7 +5273,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V14" s="26">
         <v>44.826999999999998</v>
@@ -5287,22 +5288,22 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="AC14" s="34" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD14" s="34" t="s">
         <v>408</v>
       </c>
-      <c r="AD14" s="34" t="s">
-        <v>409</v>
-      </c>
       <c r="AE14" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" spans="1:32" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5367,7 +5368,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V15" s="26">
         <v>43.186100000000003</v>
@@ -5382,20 +5383,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="16" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5418,7 +5419,7 @@
         <v>275</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5460,7 +5461,7 @@
         <v>146415990</v>
       </c>
       <c r="U16" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V16" s="24">
         <v>45.290985428950698</v>
@@ -5472,25 +5473,25 @@
         <v>244</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA16" s="30" t="s">
         <v>286</v>
       </c>
       <c r="AB16" s="46" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="AC16" s="30" t="s">
+        <v>424</v>
+      </c>
+      <c r="AD16" s="30" t="s">
         <v>425</v>
       </c>
-      <c r="AD16" s="30" t="s">
-        <v>426</v>
-      </c>
       <c r="AE16" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5513,7 +5514,7 @@
         <v>253</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5555,7 +5556,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V17" s="23">
         <v>51.870851200822599</v>
@@ -5567,10 +5568,10 @@
         <v>244</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA17" s="30" t="s">
         <v>254</v>
@@ -5579,10 +5580,10 @@
         <v>255</v>
       </c>
       <c r="AC17" s="30" t="s">
+        <v>428</v>
+      </c>
+      <c r="AD17" s="30" t="s">
         <v>429</v>
-      </c>
-      <c r="AD17" s="30" t="s">
-        <v>430</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5650,7 +5651,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V18" s="24">
         <v>52.489100000000001</v>
@@ -5665,7 +5666,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5674,13 +5675,13 @@
         <v>208</v>
       </c>
       <c r="AC18" s="30" t="s">
+        <v>384</v>
+      </c>
+      <c r="AD18" s="30" t="s">
         <v>385</v>
       </c>
-      <c r="AD18" s="30" t="s">
-        <v>386</v>
-      </c>
       <c r="AE18" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5745,7 +5746,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V19" s="26">
         <v>50.569000000000003</v>
@@ -5760,13 +5761,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5786,10 +5787,10 @@
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5798,7 +5799,7 @@
         <v>235</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5855,7 +5856,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5864,13 +5865,13 @@
         <v>240</v>
       </c>
       <c r="AC20" s="34" t="s">
+        <v>432</v>
+      </c>
+      <c r="AD20" s="34" t="s">
         <v>433</v>
       </c>
-      <c r="AD20" s="34" t="s">
-        <v>434</v>
-      </c>
       <c r="AE20" s="66" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5881,10 +5882,10 @@
         <v>302</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5923,10 +5924,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="36" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="R21" s="36" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="S21" s="22" t="s">
         <v>122</v>
@@ -5935,7 +5936,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V21" s="26">
         <v>41.352637812781921</v>
@@ -5947,25 +5948,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="Z21" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA21" s="34" t="s">
         <v>303</v>
       </c>
       <c r="AB21" s="46" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AC21" s="34" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="AD21" s="34" t="s">
         <v>304</v>
       </c>
       <c r="AE21" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6042,25 +6043,25 @@
         <v>244</v>
       </c>
       <c r="Y22" s="29" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
       <c r="AB22" s="46" t="s">
+        <v>437</v>
+      </c>
+      <c r="AC22" s="30" t="s">
         <v>438</v>
       </c>
-      <c r="AC22" s="30" t="s">
+      <c r="AD22" s="30" t="s">
         <v>439</v>
       </c>
-      <c r="AD22" s="30" t="s">
-        <v>440</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6080,10 +6081,10 @@
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6137,25 +6138,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>442</v>
+      </c>
+      <c r="AC23" s="34" t="s">
         <v>443</v>
       </c>
-      <c r="AC23" s="34" t="s">
+      <c r="AD23" s="34" t="s">
         <v>444</v>
       </c>
-      <c r="AD23" s="34" t="s">
-        <v>445</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6166,7 +6167,7 @@
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>150</v>
@@ -6175,10 +6176,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
+        <v>451</v>
+      </c>
+      <c r="G24" s="72" t="s">
         <v>452</v>
-      </c>
-      <c r="G24" s="72" t="s">
-        <v>453</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6232,25 +6233,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="AC24" s="34" t="s">
+        <v>453</v>
+      </c>
+      <c r="AD24" s="34" t="s">
         <v>454</v>
       </c>
-      <c r="AD24" s="34" t="s">
-        <v>455</v>
-      </c>
       <c r="AE24" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6270,10 +6271,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6315,7 +6316,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V25" s="26">
         <v>45.515127894849797</v>
@@ -6327,25 +6328,25 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
+        <v>587</v>
+      </c>
+      <c r="Z25" s="34" t="s">
+        <v>578</v>
+      </c>
+      <c r="AA25" s="34" t="s">
         <v>588</v>
       </c>
-      <c r="Z25" s="34" t="s">
-        <v>579</v>
-      </c>
-      <c r="AA25" s="34" t="s">
-        <v>589</v>
-      </c>
       <c r="AB25" s="46" t="s">
+        <v>447</v>
+      </c>
+      <c r="AC25" s="34" t="s">
         <v>448</v>
       </c>
-      <c r="AC25" s="34" t="s">
+      <c r="AD25" s="34" t="s">
         <v>449</v>
       </c>
-      <c r="AD25" s="34" t="s">
-        <v>450</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6356,7 +6357,7 @@
         <v>258</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6410,7 +6411,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V26" s="22">
         <v>59.121267699503399</v>
@@ -6422,10 +6423,10 @@
         <v>244</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA26" s="34" t="s">
         <v>260</v>
@@ -6434,13 +6435,13 @@
         <v>261</v>
       </c>
       <c r="AC26" s="34" t="s">
+        <v>583</v>
+      </c>
+      <c r="AD26" s="34" t="s">
         <v>584</v>
       </c>
-      <c r="AD26" s="34" t="s">
-        <v>585</v>
-      </c>
       <c r="AE26" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6463,7 +6464,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6517,10 +6518,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6529,13 +6530,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
+        <v>458</v>
+      </c>
+      <c r="AD27" s="30" t="s">
         <v>459</v>
       </c>
-      <c r="AD27" s="30" t="s">
-        <v>460</v>
-      </c>
       <c r="AE27" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6549,7 +6550,7 @@
         <v>225</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6612,25 +6613,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>462</v>
+      </c>
+      <c r="AC28" s="30" t="s">
         <v>463</v>
       </c>
-      <c r="AC28" s="30" t="s">
+      <c r="AD28" s="30" t="s">
         <v>464</v>
       </c>
-      <c r="AD28" s="30" t="s">
-        <v>465</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6695,7 +6696,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V29" s="24">
         <v>51.297800000000002</v>
@@ -6707,10 +6708,10 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6719,13 +6720,13 @@
         <v>199</v>
       </c>
       <c r="AC29" s="30" t="s">
+        <v>466</v>
+      </c>
+      <c r="AD29" s="30" t="s">
         <v>467</v>
       </c>
-      <c r="AD29" s="30" t="s">
-        <v>468</v>
-      </c>
       <c r="AE29" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6733,19 +6734,19 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>312</v>
@@ -6790,7 +6791,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V30" s="22">
         <v>60.618241659279597</v>
@@ -6802,25 +6803,25 @@
         <v>244</v>
       </c>
       <c r="Y30" s="34" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA30" s="34" t="s">
         <v>313</v>
       </c>
       <c r="AB30" s="47" t="s">
+        <v>493</v>
+      </c>
+      <c r="AC30" s="34" t="s">
         <v>494</v>
       </c>
-      <c r="AC30" s="34" t="s">
+      <c r="AD30" s="34" t="s">
         <v>495</v>
       </c>
-      <c r="AD30" s="34" t="s">
-        <v>496</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6885,7 +6886,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V31" s="26">
         <v>51.618000000000002</v>
@@ -6900,7 +6901,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -6909,13 +6910,13 @@
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
+        <v>405</v>
+      </c>
+      <c r="AD31" s="34" t="s">
         <v>406</v>
       </c>
-      <c r="AD31" s="34" t="s">
-        <v>407</v>
-      </c>
       <c r="AE31" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6935,10 +6936,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6992,25 +6993,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="Z32" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA32" s="34" t="s">
         <v>276</v>
       </c>
       <c r="AB32" s="46" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="AC32" s="34" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="AD32" s="34" t="s">
         <v>277</v>
       </c>
       <c r="AE32" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7090,22 +7091,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="AC33" s="30" t="s">
+        <v>470</v>
+      </c>
+      <c r="AD33" s="30" t="s">
         <v>471</v>
       </c>
-      <c r="AD33" s="30" t="s">
-        <v>472</v>
-      </c>
       <c r="AE33" s="66" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7119,7 +7120,7 @@
         <v>225</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
@@ -7168,7 +7169,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V34" s="23">
         <v>43.151000000000003</v>
@@ -7180,10 +7181,10 @@
         <v>244</v>
       </c>
       <c r="Y34" s="30" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="Z34" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA34" s="30" t="s">
         <v>292</v>
@@ -7192,13 +7193,13 @@
         <v>293</v>
       </c>
       <c r="AC34" s="30" t="s">
+        <v>474</v>
+      </c>
+      <c r="AD34" s="30" t="s">
         <v>475</v>
       </c>
-      <c r="AD34" s="30" t="s">
-        <v>476</v>
-      </c>
       <c r="AE34" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7209,10 +7210,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7221,7 +7222,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7278,19 +7279,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="AC35" s="34" t="s">
+        <v>370</v>
+      </c>
+      <c r="AD35" s="34" t="s">
         <v>371</v>
-      </c>
-      <c r="AD35" s="34" t="s">
-        <v>372</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7304,7 +7305,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7358,7 +7359,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V36" s="26">
         <v>51.1339349</v>
@@ -7370,25 +7371,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AC36" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="AD36" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="AD36" s="34" t="s">
-        <v>480</v>
-      </c>
       <c r="AE36" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7399,10 +7400,10 @@
         <v>281</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
@@ -7453,7 +7454,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V37" s="26">
         <v>50.529000000000003</v>
@@ -7468,22 +7469,22 @@
         <v>284</v>
       </c>
       <c r="Z37" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA37" s="34" t="s">
         <v>285</v>
       </c>
       <c r="AB37" s="46" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="AC37" s="34" t="s">
+        <v>480</v>
+      </c>
+      <c r="AD37" s="34" t="s">
         <v>481</v>
       </c>
-      <c r="AD37" s="34" t="s">
-        <v>482</v>
-      </c>
       <c r="AE37" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7548,7 +7549,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V38" s="26">
         <v>38.129899999999999</v>
@@ -7560,25 +7561,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
       <c r="AB38" s="46" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="AC38" s="34" t="s">
+        <v>401</v>
+      </c>
+      <c r="AD38" s="34" t="s">
         <v>402</v>
       </c>
-      <c r="AD38" s="34" t="s">
-        <v>403</v>
-      </c>
       <c r="AE38" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7589,7 +7590,7 @@
         <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7653,25 +7654,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA39" s="30" t="s">
         <v>311</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7685,7 +7686,7 @@
         <v>219</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -7736,7 +7737,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V40" s="24">
         <v>37.916800000000002</v>
@@ -7751,7 +7752,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7760,13 +7761,13 @@
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
+        <v>485</v>
+      </c>
+      <c r="AD40" s="30" t="s">
         <v>486</v>
       </c>
-      <c r="AD40" s="30" t="s">
-        <v>487</v>
-      </c>
       <c r="AE40" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7846,22 +7847,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="AC41" s="30" t="s">
+        <v>487</v>
+      </c>
+      <c r="AD41" s="30" t="s">
         <v>488</v>
       </c>
-      <c r="AD41" s="30" t="s">
-        <v>489</v>
-      </c>
       <c r="AE41" s="66" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7926,7 +7927,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V42" s="26">
         <v>44.968299999999999</v>
@@ -7941,22 +7942,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7964,13 +7965,13 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
+        <v>373</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>375</v>
-      </c>
       <c r="D43" s="30" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
@@ -8021,7 +8022,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V43" s="26">
         <v>51.976999999999997</v>
@@ -8036,22 +8037,22 @@
         <v>257</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>375</v>
+      </c>
+      <c r="AC43" s="34" t="s">
         <v>376</v>
       </c>
-      <c r="AC43" s="34" t="s">
+      <c r="AD43" s="34" t="s">
         <v>377</v>
       </c>
-      <c r="AD43" s="34" t="s">
-        <v>378</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8116,7 +8117,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V44" s="26">
         <v>50.406342306737002</v>
@@ -8128,25 +8129,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>497</v>
+      </c>
+      <c r="AC44" s="34" t="s">
         <v>498</v>
       </c>
-      <c r="AC44" s="34" t="s">
+      <c r="AD44" s="34" t="s">
         <v>499</v>
       </c>
-      <c r="AD44" s="34" t="s">
-        <v>500</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8157,16 +8158,16 @@
         <v>264</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8211,7 +8212,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V45" s="22">
         <v>59.2181</v>
@@ -8223,7 +8224,7 @@
         <v>244</v>
       </c>
       <c r="Y45" s="34" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="Z45" s="34" t="s">
         <v>225</v>
@@ -8232,16 +8233,16 @@
         <v>265</v>
       </c>
       <c r="AB45" s="46" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AC45" s="34" t="s">
+        <v>503</v>
+      </c>
+      <c r="AD45" s="34" t="s">
         <v>504</v>
       </c>
-      <c r="AD45" s="34" t="s">
-        <v>505</v>
-      </c>
       <c r="AE45" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8321,22 +8322,22 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
       <c r="AB46" s="46" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AC46" s="30" t="s">
+        <v>398</v>
+      </c>
+      <c r="AD46" s="30" t="s">
         <v>399</v>
       </c>
-      <c r="AD46" s="30" t="s">
-        <v>400</v>
-      </c>
       <c r="AE46" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8347,7 +8348,7 @@
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>150</v>
@@ -8356,10 +8357,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>506</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>507</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8416,22 +8417,22 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="AC47" s="30" t="s">
+        <v>507</v>
+      </c>
+      <c r="AD47" s="30" t="s">
         <v>508</v>
       </c>
-      <c r="AD47" s="30" t="s">
-        <v>509</v>
-      </c>
       <c r="AE47" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8439,7 +8440,7 @@
         <v>87</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
@@ -8451,10 +8452,10 @@
         <v>58</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8496,7 +8497,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="V48" s="22">
         <v>58.099057767351503</v>
@@ -8508,25 +8509,25 @@
         <v>244</v>
       </c>
       <c r="Y48" s="34" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA48" s="34" t="s">
         <v>308</v>
       </c>
       <c r="AB48" s="47" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="AD48" s="34" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8546,10 +8547,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8591,7 +8592,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V49" s="26">
         <v>56.787056035485499</v>
@@ -8606,22 +8607,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>513</v>
+      </c>
+      <c r="AC49" s="34" t="s">
         <v>514</v>
       </c>
-      <c r="AC49" s="34" t="s">
+      <c r="AD49" s="34" t="s">
         <v>515</v>
       </c>
-      <c r="AD49" s="34" t="s">
-        <v>516</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8635,7 +8636,7 @@
         <v>225</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
@@ -8674,7 +8675,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V50" s="26">
         <v>48.096166502584701</v>
@@ -8686,7 +8687,7 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="Z50" s="34" t="s">
         <v>225</v>
@@ -8695,16 +8696,16 @@
         <v>211</v>
       </c>
       <c r="AB50" s="46" t="s">
+        <v>517</v>
+      </c>
+      <c r="AC50" s="34" t="s">
         <v>518</v>
       </c>
-      <c r="AC50" s="34" t="s">
+      <c r="AD50" s="34" t="s">
         <v>519</v>
       </c>
-      <c r="AD50" s="34" t="s">
-        <v>520</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8724,10 +8725,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8781,25 +8782,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>521</v>
+      </c>
+      <c r="AC51" s="30" t="s">
         <v>522</v>
       </c>
-      <c r="AC51" s="30" t="s">
+      <c r="AD51" s="30" t="s">
         <v>523</v>
       </c>
-      <c r="AD51" s="30" t="s">
-        <v>524</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8864,7 +8865,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V52" s="26">
         <v>60.306100000000001</v>
@@ -8879,7 +8880,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8894,7 +8895,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8905,7 +8906,7 @@
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8917,7 +8918,7 @@
         <v>235</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8959,7 +8960,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V53" s="24">
         <v>64.037112316635401</v>
@@ -8971,22 +8972,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
       <c r="AB53" s="46" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="AC53" s="30" t="s">
+        <v>530</v>
+      </c>
+      <c r="AD53" s="30" t="s">
         <v>531</v>
-      </c>
-      <c r="AD53" s="30" t="s">
-        <v>532</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -9000,19 +9001,19 @@
         <v>272</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="G54" s="30" t="s">
         <v>533</v>
-      </c>
-      <c r="G54" s="30" t="s">
-        <v>534</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9054,7 +9055,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V54" s="24">
         <v>59.127044152710397</v>
@@ -9066,25 +9067,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA54" s="30" t="s">
         <v>273</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>534</v>
+      </c>
+      <c r="AC54" s="30" t="s">
         <v>535</v>
       </c>
-      <c r="AC54" s="30" t="s">
+      <c r="AD54" s="30" t="s">
         <v>536</v>
       </c>
-      <c r="AD54" s="30" t="s">
-        <v>537</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9095,19 +9096,19 @@
         <v>262</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9149,7 +9150,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V55" s="23">
         <v>57.788622470324199</v>
@@ -9161,23 +9162,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
         <v>263</v>
       </c>
       <c r="AC55" s="30" t="s">
+        <v>382</v>
+      </c>
+      <c r="AD55" s="30" t="s">
         <v>383</v>
       </c>
-      <c r="AD55" s="30" t="s">
-        <v>384</v>
-      </c>
       <c r="AE55" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9197,10 +9198,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>541</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>542</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9254,25 +9255,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>543</v>
+      </c>
+      <c r="AC56" s="30" t="s">
         <v>544</v>
       </c>
-      <c r="AC56" s="30" t="s">
+      <c r="AD56" s="30" t="s">
         <v>545</v>
       </c>
-      <c r="AD56" s="30" t="s">
-        <v>546</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9283,19 +9284,19 @@
         <v>299</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9337,7 +9338,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="33" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V57" s="24">
         <v>40.8482802817337</v>
@@ -9349,10 +9350,10 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="Z57" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AA57" s="30" t="s">
         <v>300</v>
@@ -9361,13 +9362,13 @@
         <v>301</v>
       </c>
       <c r="AC57" s="30" t="s">
+        <v>548</v>
+      </c>
+      <c r="AD57" s="30" t="s">
         <v>549</v>
       </c>
-      <c r="AD57" s="30" t="s">
-        <v>550</v>
-      </c>
       <c r="AE57" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9381,7 +9382,7 @@
         <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9444,7 +9445,7 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="Z58" s="30" t="s">
         <v>225</v>
@@ -9453,16 +9454,16 @@
         <v>230</v>
       </c>
       <c r="AB58" s="46" t="s">
+        <v>557</v>
+      </c>
+      <c r="AC58" s="30" t="s">
         <v>558</v>
       </c>
-      <c r="AC58" s="30" t="s">
+      <c r="AD58" s="30" t="s">
         <v>559</v>
       </c>
-      <c r="AD58" s="30" t="s">
-        <v>560</v>
-      </c>
       <c r="AE58" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9473,7 +9474,7 @@
         <v>294</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>150</v>
@@ -9539,10 +9540,10 @@
         <v>244</v>
       </c>
       <c r="Y59" s="34" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="Z59" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA59" s="34" t="s">
         <v>296</v>
@@ -9551,13 +9552,13 @@
         <v>297</v>
       </c>
       <c r="AC59" s="34" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="AD59" s="34" t="s">
         <v>298</v>
       </c>
       <c r="AE59" s="61" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9637,22 +9638,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
+        <v>552</v>
+      </c>
+      <c r="AC60" s="34" t="s">
         <v>553</v>
-      </c>
-      <c r="AC60" s="34" t="s">
-        <v>554</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9666,7 +9667,7 @@
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
@@ -9717,7 +9718,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="37" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="V61" s="26">
         <v>60.45333865137971</v>
@@ -9729,7 +9730,7 @@
         <v>244</v>
       </c>
       <c r="Y61" s="34" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="Z61" s="34" t="s">
         <v>225</v>
@@ -9738,16 +9739,16 @@
         <v>270</v>
       </c>
       <c r="AB61" s="46" t="s">
+        <v>555</v>
+      </c>
+      <c r="AC61" s="34" t="s">
         <v>556</v>
-      </c>
-      <c r="AC61" s="34" t="s">
-        <v>557</v>
       </c>
       <c r="AD61" s="34" t="s">
         <v>271</v>
       </c>
       <c r="AE61" s="65" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
   </sheetData>
@@ -9835,141 +9836,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="87" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="73" t="s">
         <v>315</v>
       </c>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="93" t="s">
         <v>316</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="83" t="s">
+      <c r="B4" s="77"/>
+      <c r="C4" s="82" t="s">
         <v>317</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87" t="s">
+      <c r="A5" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="83" t="s">
+      <c r="B5" s="77"/>
+      <c r="C5" s="82" t="s">
         <v>318</v>
       </c>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="85" t="s">
+      <c r="A6" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="82" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="86" t="s">
+      <c r="A7" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="83" t="s">
+      <c r="B7" s="77"/>
+      <c r="C7" s="82" t="s">
         <v>320</v>
       </c>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="83" t="s">
+      <c r="B8" s="77"/>
+      <c r="C8" s="82" t="s">
         <v>321</v>
       </c>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="93" t="s">
+      <c r="A9" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="83" t="s">
+      <c r="B9" s="77"/>
+      <c r="C9" s="82" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="91" t="s">
+      <c r="A10" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="83" t="s">
+      <c r="B10" s="77"/>
+      <c r="C10" s="82" t="s">
         <v>323</v>
       </c>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="78" t="s">
+      <c r="A12" s="73" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="92" t="s">
+      <c r="A13" s="84" t="s">
         <v>325</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="83" t="s">
+      <c r="B13" s="77"/>
+      <c r="C13" s="82" t="s">
         <v>326</v>
       </c>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="88" t="s">
+      <c r="A14" s="91" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="75"/>
-      <c r="C14" s="83" t="s">
+      <c r="B14" s="77"/>
+      <c r="C14" s="82" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="74"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="82" t="s">
+      <c r="A15" s="86" t="s">
         <v>329</v>
       </c>
-      <c r="B15" s="75"/>
-      <c r="C15" s="83" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="82" t="s">
         <v>330</v>
       </c>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
@@ -9984,13 +9985,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10007,6 +10001,13 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10014,6 +10015,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -10254,41 +10275,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10311,9 +10301,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 060526.xlsx 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 060526.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmeurope-my.sharepoint.com/personal/salman_muhammad_cmeurope_org/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1824" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49E2393-40B6-402C-A971-F8F37DFD2767}"/>
+  <xr:revisionPtr revIDLastSave="1825" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC06345D-F673-4916-8700-A737D48DCB1A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -693,7 +693,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="593">
   <si>
     <t>EU Innovation Fund — CCS/CCU Project Portfolio Summary</t>
   </si>
@@ -1280,9 +1280,6 @@
   </si>
   <si>
     <t>Take Kair</t>
-  </si>
-  <si>
-    <t>C2B</t>
   </si>
   <si>
     <t>Holcim GmbH</t>
@@ -3071,36 +3068,27 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3124,6 +3112,15 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3140,10 +3137,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3447,40 +3440,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3497,12 +3490,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3511,12 +3504,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="74"/>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="74"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3525,12 +3518,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3539,12 +3532,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="76"/>
+      <c r="H9" s="76"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3553,12 +3546,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="74"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="74"/>
+      <c r="C10" s="76"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
+      <c r="F10" s="76"/>
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3567,12 +3560,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3581,24 +3574,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="74"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="74"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="74"/>
+      <c r="B15" s="76"/>
+      <c r="C15" s="76"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3610,11 +3603,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="77"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="75"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3623,14 +3616,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="75" t="s">
+      <c r="C17" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="76"/>
-      <c r="E17" s="76"/>
-      <c r="F17" s="76"/>
-      <c r="G17" s="76"/>
-      <c r="H17" s="77"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="75"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3639,14 +3632,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="79" t="s">
+      <c r="C18" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="77"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="74"/>
+      <c r="H18" s="75"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3655,14 +3648,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="77"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="75"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3671,14 +3664,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="79" t="s">
+      <c r="C20" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="76"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="77"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="75"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3687,14 +3680,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="75"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3703,14 +3696,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="79" t="s">
+      <c r="C22" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="77"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="74"/>
+      <c r="F22" s="74"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="75"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3719,14 +3712,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="75" t="s">
+      <c r="C23" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="77"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="75"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3735,14 +3728,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="79" t="s">
+      <c r="C24" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="77"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="75"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3751,26 +3744,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="75" t="s">
+      <c r="C25" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="77"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="75"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="73" t="s">
+      <c r="A28" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="74"/>
-      <c r="C28" s="74"/>
-      <c r="D28" s="74"/>
-      <c r="E28" s="74"/>
-      <c r="F28" s="74"/>
-      <c r="G28" s="74"/>
-      <c r="H28" s="74"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="76"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
+      <c r="H28" s="76"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3914,12 +3907,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3936,6 +3923,12 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4023,10 +4016,10 @@
         <v>74</v>
       </c>
       <c r="Q1" s="28" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="R1" s="28" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="S1" s="28" t="s">
         <v>75</v>
@@ -4130,7 +4123,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V2" s="24">
         <v>57.062100000000001</v>
@@ -4145,22 +4138,22 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
       <c r="AB2" s="46" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AC2" s="30" t="s">
+        <v>591</v>
+      </c>
+      <c r="AD2" s="30" t="s">
         <v>592</v>
       </c>
-      <c r="AD2" s="30" t="s">
-        <v>593</v>
-      </c>
       <c r="AE2" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4168,10 +4161,10 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D3" s="34" t="s">
         <v>109</v>
@@ -4180,10 +4173,10 @@
         <v>56</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H3" s="31">
         <v>0.12330000000000001</v>
@@ -4225,7 +4218,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V3" s="24">
         <v>44.464755134852901</v>
@@ -4237,25 +4230,25 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
+        <v>388</v>
+      </c>
+      <c r="Z3" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA3" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB3" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="AC3" s="30" t="s">
         <v>389</v>
       </c>
-      <c r="Z3" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA3" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB3" s="46" t="s">
-        <v>250</v>
-      </c>
-      <c r="AC3" s="30" t="s">
+      <c r="AD3" s="30" t="s">
         <v>390</v>
       </c>
-      <c r="AD3" s="30" t="s">
-        <v>391</v>
-      </c>
       <c r="AE3" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4263,7 +4256,7 @@
         <v>98</v>
       </c>
       <c r="B4" s="54" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>108</v>
@@ -4275,10 +4268,10 @@
         <v>52</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H4" s="35" t="s">
         <v>92</v>
@@ -4320,7 +4313,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V4" s="26">
         <v>43.327720234653299</v>
@@ -4332,22 +4325,22 @@
         <v>95</v>
       </c>
       <c r="Y4" s="34" t="s">
+        <v>336</v>
+      </c>
+      <c r="Z4" s="34" t="s">
+        <v>578</v>
+      </c>
+      <c r="AA4" s="34" t="s">
+        <v>288</v>
+      </c>
+      <c r="AB4" s="46" t="s">
+        <v>345</v>
+      </c>
+      <c r="AC4" s="34" t="s">
         <v>337</v>
       </c>
-      <c r="Z4" s="34" t="s">
-        <v>579</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>289</v>
-      </c>
-      <c r="AB4" s="46" t="s">
-        <v>346</v>
-      </c>
-      <c r="AC4" s="34" t="s">
+      <c r="AD4" s="34" t="s">
         <v>338</v>
-      </c>
-      <c r="AD4" s="34" t="s">
-        <v>339</v>
       </c>
       <c r="AE4" s="62" t="s">
         <v>27</v>
@@ -4358,13 +4351,13 @@
         <v>119</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4400,7 +4393,7 @@
         <v>92</v>
       </c>
       <c r="P5" s="32" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q5" s="32">
         <v>2030</v>
@@ -4415,7 +4408,7 @@
         <v>170000000</v>
       </c>
       <c r="U5" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V5" s="24">
         <v>46.809800000000003</v>
@@ -4430,22 +4423,22 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
       <c r="AB5" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="AC5" s="30" t="s">
         <v>351</v>
       </c>
-      <c r="AC5" s="30" t="s">
+      <c r="AD5" s="30" t="s">
         <v>352</v>
       </c>
-      <c r="AD5" s="30" t="s">
-        <v>353</v>
-      </c>
       <c r="AE5" s="63" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="6" spans="1:32" ht="125.4" x14ac:dyDescent="0.3">
@@ -4453,10 +4446,10 @@
         <v>141</v>
       </c>
       <c r="B6" s="55" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D6" s="30" t="s">
         <v>150</v>
@@ -4465,10 +4458,10 @@
         <v>45</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H6" s="31">
         <v>2.5999999999999999E-2</v>
@@ -4510,7 +4503,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V6" s="23" t="s">
         <v>92</v>
@@ -4519,28 +4512,28 @@
         <v>92</v>
       </c>
       <c r="X6" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y6" s="30" t="s">
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA6" s="30" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AB6" s="46" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4605,7 +4598,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V7" s="24">
         <v>43.232830995956597</v>
@@ -4617,28 +4610,28 @@
         <v>132</v>
       </c>
       <c r="Y7" s="30" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
       <c r="AB7" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="AC7" s="30" t="s">
+        <v>357</v>
+      </c>
+      <c r="AD7" s="30" t="s">
         <v>359</v>
       </c>
-      <c r="AC7" s="30" t="s">
-        <v>358</v>
-      </c>
-      <c r="AD7" s="30" t="s">
-        <v>360</v>
-      </c>
       <c r="AE7" s="63" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AF7" s="29" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -4688,7 +4681,7 @@
         <v>92</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="Q8" s="32">
         <v>2029</v>
@@ -4703,7 +4696,7 @@
         <v>115000000</v>
       </c>
       <c r="U8" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V8" s="24">
         <v>50.575420999999999</v>
@@ -4718,22 +4711,22 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AE8" s="63" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="91.2" x14ac:dyDescent="0.3">
@@ -4741,22 +4734,22 @@
         <v>119</v>
       </c>
       <c r="B9" s="54" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4798,7 +4791,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V9" s="26">
         <v>37.960247145532399</v>
@@ -4810,25 +4803,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
+        <v>568</v>
+      </c>
+      <c r="Z9" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="AA9" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB9" s="46" t="s">
+        <v>363</v>
+      </c>
+      <c r="AC9" s="34" t="s">
         <v>569</v>
       </c>
-      <c r="Z9" s="34" t="s">
-        <v>580</v>
-      </c>
-      <c r="AA9" s="34" t="s">
+      <c r="AD9" s="34" t="s">
         <v>226</v>
       </c>
-      <c r="AB9" s="46" t="s">
-        <v>364</v>
-      </c>
-      <c r="AC9" s="34" t="s">
-        <v>570</v>
-      </c>
-      <c r="AD9" s="34" t="s">
-        <v>227</v>
-      </c>
       <c r="AE9" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="10" spans="1:32" ht="114" x14ac:dyDescent="0.3">
@@ -4836,22 +4829,22 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>92</v>
@@ -4905,22 +4898,22 @@
         <v>95</v>
       </c>
       <c r="Y10" s="30" t="s">
+        <v>305</v>
+      </c>
+      <c r="Z10" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA10" s="30" t="s">
         <v>306</v>
       </c>
-      <c r="Z10" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA10" s="30" t="s">
-        <v>307</v>
-      </c>
       <c r="AB10" s="46" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4931,10 +4924,10 @@
         <v>126</v>
       </c>
       <c r="B11" s="55" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>150</v>
@@ -4943,10 +4936,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4988,7 +4981,7 @@
         <v>10206000</v>
       </c>
       <c r="U11" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V11" s="24">
         <v>59.592303479664103</v>
@@ -4997,28 +4990,28 @@
         <v>5.8029778441568904</v>
       </c>
       <c r="X11" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y11" s="30" t="s">
+        <v>416</v>
+      </c>
+      <c r="Z11" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA11" s="30" t="s">
+        <v>266</v>
+      </c>
+      <c r="AB11" s="46" t="s">
+        <v>413</v>
+      </c>
+      <c r="AC11" s="30" t="s">
         <v>417</v>
       </c>
-      <c r="Z11" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA11" s="30" t="s">
-        <v>267</v>
-      </c>
-      <c r="AB11" s="46" t="s">
-        <v>414</v>
-      </c>
-      <c r="AC11" s="30" t="s">
+      <c r="AD11" s="30" t="s">
         <v>418</v>
       </c>
-      <c r="AD11" s="30" t="s">
-        <v>419</v>
-      </c>
       <c r="AE11" s="63" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5026,7 +5019,7 @@
         <v>87</v>
       </c>
       <c r="B12" s="54" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>108</v>
@@ -5038,7 +5031,7 @@
         <v>48</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>175</v>
@@ -5095,25 +5088,25 @@
         <v>95</v>
       </c>
       <c r="Y12" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="Z12" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA12" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="Z12" s="34" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA12" s="34" t="s">
-        <v>195</v>
-      </c>
       <c r="AB12" s="46" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AC12" s="34" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AE12" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5190,10 +5183,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5202,13 +5195,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
+        <v>378</v>
+      </c>
+      <c r="AD13" s="34" t="s">
         <v>379</v>
       </c>
-      <c r="AD13" s="34" t="s">
-        <v>380</v>
-      </c>
       <c r="AE13" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="14" spans="1:32" ht="79.8" x14ac:dyDescent="0.3">
@@ -5216,10 +5209,10 @@
         <v>141</v>
       </c>
       <c r="B14" s="54" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5228,10 +5221,10 @@
         <v>56</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H14" s="35">
         <v>6.4000000000000001E-2</v>
@@ -5273,7 +5266,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V14" s="26">
         <v>44.826999999999998</v>
@@ -5285,25 +5278,25 @@
         <v>180</v>
       </c>
       <c r="Y14" s="34" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AC14" s="34" t="s">
+        <v>406</v>
+      </c>
+      <c r="AD14" s="34" t="s">
         <v>407</v>
       </c>
-      <c r="AD14" s="34" t="s">
-        <v>408</v>
-      </c>
       <c r="AE14" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="15" spans="1:32" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5368,7 +5361,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V15" s="26">
         <v>43.186100000000003</v>
@@ -5383,20 +5376,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="16" spans="1:32" ht="102.6" x14ac:dyDescent="0.3">
@@ -5404,7 +5397,7 @@
         <v>119</v>
       </c>
       <c r="B16" s="55" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>108</v>
@@ -5416,10 +5409,10 @@
         <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5461,7 +5454,7 @@
         <v>146415990</v>
       </c>
       <c r="U16" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V16" s="24">
         <v>45.290985428950698</v>
@@ -5470,28 +5463,28 @@
         <v>25.1109549184484</v>
       </c>
       <c r="X16" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA16" s="30" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AB16" s="46" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC16" s="30" t="s">
+        <v>423</v>
+      </c>
+      <c r="AD16" s="30" t="s">
         <v>424</v>
       </c>
-      <c r="AD16" s="30" t="s">
-        <v>425</v>
-      </c>
       <c r="AE16" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5499,10 +5492,10 @@
         <v>98</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D17" s="30" t="s">
         <v>109</v>
@@ -5511,10 +5504,10 @@
         <v>43</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5556,7 +5549,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V17" s="23">
         <v>51.870851200822599</v>
@@ -5565,25 +5558,25 @@
         <v>4.30094696894741</v>
       </c>
       <c r="X17" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA17" s="30" t="s">
+        <v>253</v>
+      </c>
+      <c r="AB17" s="25" t="s">
         <v>254</v>
       </c>
-      <c r="AB17" s="25" t="s">
-        <v>255</v>
-      </c>
       <c r="AC17" s="30" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD17" s="30" t="s">
         <v>428</v>
-      </c>
-      <c r="AD17" s="30" t="s">
-        <v>429</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5594,7 +5587,7 @@
         <v>87</v>
       </c>
       <c r="B18" s="55" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>108</v>
@@ -5606,10 +5599,10 @@
         <v>48</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H18" s="40">
         <v>1.3</v>
@@ -5651,7 +5644,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V18" s="24">
         <v>52.489100000000001</v>
@@ -5663,25 +5656,25 @@
         <v>95</v>
       </c>
       <c r="Y18" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="Z18" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA18" s="30" t="s">
         <v>206</v>
       </c>
-      <c r="Z18" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA18" s="30" t="s">
+      <c r="AB18" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="AB18" s="25" t="s">
-        <v>208</v>
-      </c>
       <c r="AC18" s="30" t="s">
+        <v>383</v>
+      </c>
+      <c r="AD18" s="30" t="s">
         <v>384</v>
       </c>
-      <c r="AD18" s="30" t="s">
-        <v>385</v>
-      </c>
       <c r="AE18" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5746,7 +5739,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V19" s="26">
         <v>50.569000000000003</v>
@@ -5761,13 +5754,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5784,22 +5777,22 @@
         <v>87</v>
       </c>
       <c r="B20" s="54" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5853,25 +5846,25 @@
         <v>95</v>
       </c>
       <c r="Y20" s="34" t="s">
+        <v>237</v>
+      </c>
+      <c r="Z20" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="AA20" s="34" t="s">
         <v>238</v>
       </c>
-      <c r="Z20" s="34" t="s">
-        <v>580</v>
-      </c>
-      <c r="AA20" s="34" t="s">
+      <c r="AB20" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="AB20" s="27" t="s">
-        <v>240</v>
-      </c>
       <c r="AC20" s="34" t="s">
+        <v>431</v>
+      </c>
+      <c r="AD20" s="34" t="s">
         <v>432</v>
       </c>
-      <c r="AD20" s="34" t="s">
-        <v>433</v>
-      </c>
       <c r="AE20" s="66" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5879,13 +5872,13 @@
         <v>126</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5924,10 +5917,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="36" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="R21" s="36" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="S21" s="22" t="s">
         <v>122</v>
@@ -5936,7 +5929,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V21" s="26">
         <v>41.352637812781921</v>
@@ -5948,25 +5941,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
+        <v>433</v>
+      </c>
+      <c r="Z21" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="AA21" s="34" t="s">
+        <v>302</v>
+      </c>
+      <c r="AB21" s="46" t="s">
+        <v>435</v>
+      </c>
+      <c r="AC21" s="34" t="s">
         <v>434</v>
       </c>
-      <c r="Z21" s="34" t="s">
-        <v>580</v>
-      </c>
-      <c r="AA21" s="34" t="s">
+      <c r="AD21" s="34" t="s">
         <v>303</v>
       </c>
-      <c r="AB21" s="46" t="s">
-        <v>436</v>
-      </c>
-      <c r="AC21" s="34" t="s">
-        <v>435</v>
-      </c>
-      <c r="AD21" s="34" t="s">
-        <v>304</v>
-      </c>
       <c r="AE21" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5974,10 +5967,10 @@
         <v>98</v>
       </c>
       <c r="B22" s="55" t="s">
+        <v>240</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>242</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>150</v>
@@ -5986,10 +5979,10 @@
         <v>56</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H22" s="52">
         <v>1.7904E-2</v>
@@ -6040,28 +6033,28 @@
         <v>13.253440646806</v>
       </c>
       <c r="X22" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="Y22" s="29" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z22" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA22" s="30" t="s">
         <v>244</v>
       </c>
-      <c r="Y22" s="29" t="s">
-        <v>440</v>
-      </c>
-      <c r="Z22" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA22" s="30" t="s">
-        <v>245</v>
-      </c>
       <c r="AB22" s="46" t="s">
+        <v>436</v>
+      </c>
+      <c r="AC22" s="30" t="s">
         <v>437</v>
       </c>
-      <c r="AC22" s="30" t="s">
+      <c r="AD22" s="30" t="s">
         <v>438</v>
       </c>
-      <c r="AD22" s="30" t="s">
-        <v>439</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6069,22 +6062,22 @@
         <v>141</v>
       </c>
       <c r="B23" s="54" t="s">
+        <v>230</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="D23" s="34" t="s">
         <v>231</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="D23" s="34" t="s">
-        <v>232</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6138,25 +6131,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA23" s="34" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>441</v>
+      </c>
+      <c r="AC23" s="34" t="s">
         <v>442</v>
       </c>
-      <c r="AC23" s="34" t="s">
+      <c r="AD23" s="34" t="s">
         <v>443</v>
       </c>
-      <c r="AD23" s="34" t="s">
-        <v>444</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6167,7 +6160,7 @@
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>150</v>
@@ -6176,10 +6169,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
+        <v>450</v>
+      </c>
+      <c r="G24" s="72" t="s">
         <v>451</v>
-      </c>
-      <c r="G24" s="72" t="s">
-        <v>452</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6233,25 +6226,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="AC24" s="34" t="s">
+        <v>452</v>
+      </c>
+      <c r="AD24" s="34" t="s">
         <v>453</v>
       </c>
-      <c r="AD24" s="34" t="s">
-        <v>454</v>
-      </c>
       <c r="AE24" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6259,7 +6252,7 @@
         <v>119</v>
       </c>
       <c r="B25" s="54" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>108</v>
@@ -6271,10 +6264,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6316,7 +6309,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V25" s="26">
         <v>45.515127894849797</v>
@@ -6325,28 +6318,28 @@
         <v>10.343124922954001</v>
       </c>
       <c r="X25" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y25" s="34" t="s">
+        <v>586</v>
+      </c>
+      <c r="Z25" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA25" s="34" t="s">
         <v>587</v>
       </c>
-      <c r="Z25" s="34" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA25" s="34" t="s">
-        <v>588</v>
-      </c>
       <c r="AB25" s="46" t="s">
+        <v>446</v>
+      </c>
+      <c r="AC25" s="34" t="s">
         <v>447</v>
       </c>
-      <c r="AC25" s="34" t="s">
+      <c r="AD25" s="34" t="s">
         <v>448</v>
       </c>
-      <c r="AD25" s="34" t="s">
-        <v>449</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6354,10 +6347,10 @@
         <v>87</v>
       </c>
       <c r="B26" s="54" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6366,7 +6359,7 @@
         <v>46</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>93</v>
@@ -6411,7 +6404,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V26" s="22">
         <v>59.121267699503399</v>
@@ -6420,28 +6413,28 @@
         <v>9.6300609243118291</v>
       </c>
       <c r="X26" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA26" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="AB26" s="27" t="s">
         <v>260</v>
       </c>
-      <c r="AB26" s="27" t="s">
-        <v>261</v>
-      </c>
       <c r="AC26" s="34" t="s">
+        <v>582</v>
+      </c>
+      <c r="AD26" s="34" t="s">
         <v>583</v>
       </c>
-      <c r="AD26" s="34" t="s">
-        <v>584</v>
-      </c>
       <c r="AE26" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6464,7 +6457,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6518,10 +6511,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6530,13 +6523,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
+        <v>457</v>
+      </c>
+      <c r="AD27" s="30" t="s">
         <v>458</v>
       </c>
-      <c r="AD27" s="30" t="s">
-        <v>459</v>
-      </c>
       <c r="AE27" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6547,10 +6540,10 @@
         <v>146</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6613,25 +6606,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>461</v>
+      </c>
+      <c r="AC28" s="30" t="s">
         <v>462</v>
       </c>
-      <c r="AC28" s="30" t="s">
+      <c r="AD28" s="30" t="s">
         <v>463</v>
       </c>
-      <c r="AD28" s="30" t="s">
-        <v>464</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6639,7 +6632,7 @@
         <v>87</v>
       </c>
       <c r="B29" s="55" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>100</v>
@@ -6651,10 +6644,10 @@
         <v>48</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H29" s="40">
         <v>1.5</v>
@@ -6696,7 +6689,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V29" s="24">
         <v>51.297800000000002</v>
@@ -6708,25 +6701,25 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
+        <v>464</v>
+      </c>
+      <c r="Z29" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA29" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="AB29" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="AC29" s="30" t="s">
         <v>465</v>
       </c>
-      <c r="Z29" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA29" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="AB29" s="25" t="s">
-        <v>199</v>
-      </c>
-      <c r="AC29" s="30" t="s">
+      <c r="AD29" s="30" t="s">
         <v>466</v>
       </c>
-      <c r="AD29" s="30" t="s">
-        <v>467</v>
-      </c>
       <c r="AE29" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6734,22 +6727,22 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H30" s="53">
         <v>4.5999999999999999E-2</v>
@@ -6791,7 +6784,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V30" s="22">
         <v>60.618241659279597</v>
@@ -6800,28 +6793,28 @@
         <v>16.891107915855802</v>
       </c>
       <c r="X30" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y30" s="34" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA30" s="34" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="AB30" s="47" t="s">
+        <v>492</v>
+      </c>
+      <c r="AC30" s="34" t="s">
         <v>493</v>
       </c>
-      <c r="AC30" s="34" t="s">
+      <c r="AD30" s="34" t="s">
         <v>494</v>
       </c>
-      <c r="AD30" s="34" t="s">
-        <v>495</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6829,7 +6822,7 @@
         <v>87</v>
       </c>
       <c r="B31" s="54" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>108</v>
@@ -6886,7 +6879,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V31" s="26">
         <v>51.618000000000002</v>
@@ -6898,25 +6891,25 @@
         <v>95</v>
       </c>
       <c r="Y31" s="34" t="s">
+        <v>200</v>
+      </c>
+      <c r="Z31" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA31" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="Z31" s="34" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA31" s="34" t="s">
+      <c r="AB31" s="70" t="s">
         <v>202</v>
       </c>
-      <c r="AB31" s="70" t="s">
-        <v>203</v>
-      </c>
       <c r="AC31" s="34" t="s">
+        <v>404</v>
+      </c>
+      <c r="AD31" s="34" t="s">
         <v>405</v>
       </c>
-      <c r="AD31" s="34" t="s">
-        <v>406</v>
-      </c>
       <c r="AE31" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6924,7 +6917,7 @@
         <v>87</v>
       </c>
       <c r="B32" s="54" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>108</v>
@@ -6936,10 +6929,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6993,25 +6986,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
+        <v>467</v>
+      </c>
+      <c r="Z32" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA32" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="AB32" s="46" t="s">
         <v>468</v>
       </c>
-      <c r="Z32" s="34" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA32" s="34" t="s">
+      <c r="AC32" s="34" t="s">
+        <v>386</v>
+      </c>
+      <c r="AD32" s="34" t="s">
         <v>276</v>
       </c>
-      <c r="AB32" s="46" t="s">
-        <v>469</v>
-      </c>
-      <c r="AC32" s="34" t="s">
-        <v>387</v>
-      </c>
-      <c r="AD32" s="34" t="s">
-        <v>277</v>
-      </c>
       <c r="AE32" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7091,22 +7084,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="AC33" s="30" t="s">
+        <v>469</v>
+      </c>
+      <c r="AD33" s="30" t="s">
         <v>470</v>
       </c>
-      <c r="AD33" s="30" t="s">
-        <v>471</v>
-      </c>
       <c r="AE33" s="66" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7114,19 +7107,19 @@
         <v>87</v>
       </c>
       <c r="B34" s="55" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="31">
@@ -7169,7 +7162,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V34" s="23">
         <v>43.151000000000003</v>
@@ -7178,28 +7171,28 @@
         <v>-7.6859999999999999</v>
       </c>
       <c r="X34" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y34" s="30" t="s">
+        <v>472</v>
+      </c>
+      <c r="Z34" s="30" t="s">
+        <v>580</v>
+      </c>
+      <c r="AA34" s="30" t="s">
+        <v>291</v>
+      </c>
+      <c r="AB34" s="46" t="s">
+        <v>292</v>
+      </c>
+      <c r="AC34" s="30" t="s">
         <v>473</v>
       </c>
-      <c r="Z34" s="30" t="s">
-        <v>581</v>
-      </c>
-      <c r="AA34" s="30" t="s">
-        <v>292</v>
-      </c>
-      <c r="AB34" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="AC34" s="30" t="s">
+      <c r="AD34" s="30" t="s">
         <v>474</v>
       </c>
-      <c r="AD34" s="30" t="s">
-        <v>475</v>
-      </c>
       <c r="AE34" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7210,10 +7203,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7222,7 +7215,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7279,19 +7272,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AC35" s="34" t="s">
+        <v>369</v>
+      </c>
+      <c r="AD35" s="34" t="s">
         <v>370</v>
-      </c>
-      <c r="AD35" s="34" t="s">
-        <v>371</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7305,7 +7298,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7359,7 +7352,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V36" s="26">
         <v>51.1339349</v>
@@ -7371,25 +7364,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="AC36" s="34" t="s">
+        <v>477</v>
+      </c>
+      <c r="AD36" s="34" t="s">
         <v>478</v>
       </c>
-      <c r="AD36" s="34" t="s">
-        <v>479</v>
-      </c>
       <c r="AE36" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7397,22 +7390,22 @@
         <v>163</v>
       </c>
       <c r="B37" s="54" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
       </c>
       <c r="F37" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>282</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>283</v>
       </c>
       <c r="H37" s="53">
         <v>5.0046999999999999E-3</v>
@@ -7454,7 +7447,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V37" s="26">
         <v>50.529000000000003</v>
@@ -7466,25 +7459,25 @@
         <v>95</v>
       </c>
       <c r="Y37" s="34" t="s">
+        <v>283</v>
+      </c>
+      <c r="Z37" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="AA37" s="34" t="s">
         <v>284</v>
       </c>
-      <c r="Z37" s="34" t="s">
-        <v>580</v>
-      </c>
-      <c r="AA37" s="34" t="s">
-        <v>285</v>
-      </c>
       <c r="AB37" s="46" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AC37" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="AD37" s="34" t="s">
         <v>480</v>
       </c>
-      <c r="AD37" s="34" t="s">
-        <v>481</v>
-      </c>
       <c r="AE37" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7492,7 +7485,7 @@
         <v>87</v>
       </c>
       <c r="B38" s="54" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>108</v>
@@ -7504,10 +7497,10 @@
         <v>50</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H38" s="35">
         <v>0.68</v>
@@ -7549,7 +7542,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V38" s="26">
         <v>38.129899999999999</v>
@@ -7561,25 +7554,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
+        <v>402</v>
+      </c>
+      <c r="Z38" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA38" s="34" t="s">
+        <v>216</v>
+      </c>
+      <c r="AB38" s="46" t="s">
         <v>403</v>
       </c>
-      <c r="Z38" s="34" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA38" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="AB38" s="46" t="s">
-        <v>404</v>
-      </c>
       <c r="AC38" s="34" t="s">
+        <v>400</v>
+      </c>
+      <c r="AD38" s="34" t="s">
         <v>401</v>
       </c>
-      <c r="AD38" s="34" t="s">
-        <v>402</v>
-      </c>
       <c r="AE38" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7587,10 +7580,10 @@
         <v>141</v>
       </c>
       <c r="B39" s="55" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7599,7 +7592,7 @@
         <v>58</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="31">
@@ -7654,25 +7647,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA39" s="30" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7680,22 +7673,22 @@
         <v>87</v>
       </c>
       <c r="B40" s="55" t="s">
+        <v>217</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="D40" s="30" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H40" s="31">
         <v>0.85799999999999998</v>
@@ -7737,7 +7730,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V40" s="24">
         <v>37.916800000000002</v>
@@ -7749,25 +7742,25 @@
         <v>95</v>
       </c>
       <c r="Y40" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="Z40" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA40" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="Z40" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA40" s="30" t="s">
+      <c r="AB40" s="46" t="s">
         <v>222</v>
       </c>
-      <c r="AB40" s="46" t="s">
-        <v>223</v>
-      </c>
       <c r="AC40" s="30" t="s">
+        <v>484</v>
+      </c>
+      <c r="AD40" s="30" t="s">
         <v>485</v>
       </c>
-      <c r="AD40" s="30" t="s">
-        <v>486</v>
-      </c>
       <c r="AE40" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7847,22 +7840,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AC41" s="30" t="s">
+        <v>486</v>
+      </c>
+      <c r="AD41" s="30" t="s">
         <v>487</v>
       </c>
-      <c r="AD41" s="30" t="s">
-        <v>488</v>
-      </c>
       <c r="AE41" s="66" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7927,7 +7920,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V42" s="26">
         <v>44.968299999999999</v>
@@ -7942,22 +7935,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7965,19 +7958,19 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
+        <v>372</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>374</v>
-      </c>
       <c r="D43" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G43" s="4" t="s">
         <v>92</v>
@@ -8022,7 +8015,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V43" s="26">
         <v>51.976999999999997</v>
@@ -8034,25 +8027,25 @@
         <v>95</v>
       </c>
       <c r="Y43" s="34" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>374</v>
+      </c>
+      <c r="AC43" s="34" t="s">
         <v>375</v>
       </c>
-      <c r="AC43" s="34" t="s">
+      <c r="AD43" s="34" t="s">
         <v>376</v>
       </c>
-      <c r="AD43" s="34" t="s">
-        <v>377</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8117,7 +8110,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V44" s="26">
         <v>50.406342306737002</v>
@@ -8129,25 +8122,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>496</v>
+      </c>
+      <c r="AC44" s="34" t="s">
         <v>497</v>
       </c>
-      <c r="AC44" s="34" t="s">
+      <c r="AD44" s="34" t="s">
         <v>498</v>
       </c>
-      <c r="AD44" s="34" t="s">
-        <v>499</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8155,19 +8148,19 @@
         <v>163</v>
       </c>
       <c r="B45" s="54" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8212,7 +8205,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V45" s="22">
         <v>59.2181</v>
@@ -8221,28 +8214,28 @@
         <v>10.9298</v>
       </c>
       <c r="X45" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y45" s="34" t="s">
+        <v>501</v>
+      </c>
+      <c r="Z45" s="34" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA45" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="AB45" s="46" t="s">
+        <v>499</v>
+      </c>
+      <c r="AC45" s="34" t="s">
         <v>502</v>
       </c>
-      <c r="Z45" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="AA45" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="AB45" s="46" t="s">
-        <v>500</v>
-      </c>
-      <c r="AC45" s="34" t="s">
+      <c r="AD45" s="34" t="s">
         <v>503</v>
       </c>
-      <c r="AD45" s="34" t="s">
-        <v>504</v>
-      </c>
       <c r="AE45" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8250,7 +8243,7 @@
         <v>87</v>
       </c>
       <c r="B46" s="56" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>108</v>
@@ -8262,7 +8255,7 @@
         <v>50</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>175</v>
@@ -8319,25 +8312,25 @@
         <v>95</v>
       </c>
       <c r="Y46" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="Z46" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA46" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="Z46" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA46" s="30" t="s">
-        <v>215</v>
-      </c>
       <c r="AB46" s="46" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AC46" s="30" t="s">
+        <v>397</v>
+      </c>
+      <c r="AD46" s="30" t="s">
         <v>398</v>
       </c>
-      <c r="AD46" s="30" t="s">
-        <v>399</v>
-      </c>
       <c r="AE46" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8348,7 +8341,7 @@
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>150</v>
@@ -8357,10 +8350,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>505</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>506</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8417,22 +8410,22 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AC47" s="30" t="s">
+        <v>506</v>
+      </c>
+      <c r="AD47" s="30" t="s">
         <v>507</v>
       </c>
-      <c r="AD47" s="30" t="s">
-        <v>508</v>
-      </c>
       <c r="AE47" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8440,7 +8433,7 @@
         <v>87</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
@@ -8452,10 +8445,10 @@
         <v>58</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8497,7 +8490,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="V48" s="22">
         <v>58.099057767351503</v>
@@ -8506,28 +8499,28 @@
         <v>11.861499508001399</v>
       </c>
       <c r="X48" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y48" s="34" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA48" s="34" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AB48" s="47" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="AD48" s="34" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8538,7 +8531,7 @@
         <v>149</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D49" s="34" t="s">
         <v>150</v>
@@ -8547,10 +8540,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8592,7 +8585,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V49" s="26">
         <v>56.787056035485499</v>
@@ -8607,22 +8600,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>512</v>
+      </c>
+      <c r="AC49" s="34" t="s">
         <v>513</v>
       </c>
-      <c r="AC49" s="34" t="s">
+      <c r="AD49" s="34" t="s">
         <v>514</v>
       </c>
-      <c r="AD49" s="34" t="s">
-        <v>515</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8630,22 +8623,22 @@
         <v>126</v>
       </c>
       <c r="B50" s="54" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C50" s="34" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H50" s="35">
         <v>0.24099999999999999</v>
@@ -8675,7 +8668,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V50" s="26">
         <v>48.096166502584701</v>
@@ -8687,25 +8680,25 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
+        <v>515</v>
+      </c>
+      <c r="Z50" s="34" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA50" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB50" s="46" t="s">
         <v>516</v>
       </c>
-      <c r="Z50" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="AA50" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="AB50" s="46" t="s">
+      <c r="AC50" s="34" t="s">
         <v>517</v>
       </c>
-      <c r="AC50" s="34" t="s">
+      <c r="AD50" s="34" t="s">
         <v>518</v>
       </c>
-      <c r="AD50" s="34" t="s">
-        <v>519</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8716,7 +8709,7 @@
         <v>182</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>150</v>
@@ -8725,10 +8718,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8782,25 +8775,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>520</v>
+      </c>
+      <c r="AC51" s="30" t="s">
         <v>521</v>
       </c>
-      <c r="AC51" s="30" t="s">
+      <c r="AD51" s="30" t="s">
         <v>522</v>
       </c>
-      <c r="AD51" s="30" t="s">
-        <v>523</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8811,7 +8804,7 @@
         <v>156</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>109</v>
@@ -8865,7 +8858,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V52" s="26">
         <v>60.306100000000001</v>
@@ -8880,7 +8873,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8895,7 +8888,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8903,10 +8896,10 @@
         <v>98</v>
       </c>
       <c r="B53" s="55" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8915,10 +8908,10 @@
         <v>49</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8960,7 +8953,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V53" s="24">
         <v>64.037112316635401</v>
@@ -8972,22 +8965,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
+        <v>526</v>
+      </c>
+      <c r="Z53" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="AA53" s="30" t="s">
+        <v>235</v>
+      </c>
+      <c r="AB53" s="46" t="s">
         <v>527</v>
       </c>
-      <c r="Z53" s="30" t="s">
-        <v>578</v>
-      </c>
-      <c r="AA53" s="30" t="s">
-        <v>236</v>
-      </c>
-      <c r="AB53" s="46" t="s">
-        <v>528</v>
-      </c>
       <c r="AC53" s="30" t="s">
+        <v>529</v>
+      </c>
+      <c r="AD53" s="30" t="s">
         <v>530</v>
-      </c>
-      <c r="AD53" s="30" t="s">
-        <v>531</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -8998,22 +8991,22 @@
         <v>163</v>
       </c>
       <c r="B54" s="55" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="G54" s="30" t="s">
         <v>532</v>
-      </c>
-      <c r="G54" s="30" t="s">
-        <v>533</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9055,7 +9048,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V54" s="24">
         <v>59.127044152710397</v>
@@ -9067,25 +9060,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA54" s="30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>533</v>
+      </c>
+      <c r="AC54" s="30" t="s">
         <v>534</v>
       </c>
-      <c r="AC54" s="30" t="s">
+      <c r="AD54" s="30" t="s">
         <v>535</v>
       </c>
-      <c r="AD54" s="30" t="s">
-        <v>536</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9093,22 +9086,22 @@
         <v>87</v>
       </c>
       <c r="B55" s="55" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9150,7 +9143,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V55" s="23">
         <v>57.788622470324199</v>
@@ -9162,23 +9155,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="AC55" s="30" t="s">
+        <v>381</v>
+      </c>
+      <c r="AD55" s="30" t="s">
         <v>382</v>
       </c>
-      <c r="AD55" s="30" t="s">
-        <v>383</v>
-      </c>
       <c r="AE55" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9198,10 +9191,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>540</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>541</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9255,25 +9248,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>542</v>
+      </c>
+      <c r="AC56" s="30" t="s">
         <v>543</v>
       </c>
-      <c r="AC56" s="30" t="s">
+      <c r="AD56" s="30" t="s">
         <v>544</v>
       </c>
-      <c r="AD56" s="30" t="s">
-        <v>545</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9281,22 +9274,22 @@
         <v>87</v>
       </c>
       <c r="B57" s="55" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9338,7 +9331,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V57" s="24">
         <v>40.8482802817337</v>
@@ -9350,25 +9343,25 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
+        <v>546</v>
+      </c>
+      <c r="Z57" s="30" t="s">
+        <v>581</v>
+      </c>
+      <c r="AA57" s="30" t="s">
+        <v>299</v>
+      </c>
+      <c r="AB57" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="AC57" s="30" t="s">
         <v>547</v>
       </c>
-      <c r="Z57" s="30" t="s">
-        <v>582</v>
-      </c>
-      <c r="AA57" s="30" t="s">
-        <v>300</v>
-      </c>
-      <c r="AB57" s="25" t="s">
-        <v>301</v>
-      </c>
-      <c r="AC57" s="30" t="s">
+      <c r="AD57" s="30" t="s">
         <v>548</v>
       </c>
-      <c r="AD57" s="30" t="s">
-        <v>549</v>
-      </c>
       <c r="AE57" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9376,22 +9369,22 @@
         <v>126</v>
       </c>
       <c r="B58" s="55" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H58" s="52">
         <v>7.8E-2</v>
@@ -9445,25 +9438,25 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
+        <v>559</v>
+      </c>
+      <c r="Z58" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA58" s="30" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB58" s="46" t="s">
+        <v>556</v>
+      </c>
+      <c r="AC58" s="30" t="s">
+        <v>557</v>
+      </c>
+      <c r="AD58" s="30" t="s">
+        <v>558</v>
+      </c>
+      <c r="AE58" s="60" t="s">
         <v>560</v>
-      </c>
-      <c r="Z58" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="AA58" s="30" t="s">
-        <v>230</v>
-      </c>
-      <c r="AB58" s="46" t="s">
-        <v>557</v>
-      </c>
-      <c r="AC58" s="30" t="s">
-        <v>558</v>
-      </c>
-      <c r="AD58" s="30" t="s">
-        <v>559</v>
-      </c>
-      <c r="AE58" s="60" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9471,10 +9464,10 @@
         <v>87</v>
       </c>
       <c r="B59" s="54" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>150</v>
@@ -9483,10 +9476,10 @@
         <v>52</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H59" s="53">
         <v>8.5999999999999993E-2</v>
@@ -9537,28 +9530,28 @@
         <v>-8.2351799999999997</v>
       </c>
       <c r="X59" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y59" s="34" t="s">
+        <v>549</v>
+      </c>
+      <c r="Z59" s="34" t="s">
+        <v>580</v>
+      </c>
+      <c r="AA59" s="34" t="s">
+        <v>295</v>
+      </c>
+      <c r="AB59" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="AC59" s="34" t="s">
         <v>550</v>
       </c>
-      <c r="Z59" s="34" t="s">
-        <v>581</v>
-      </c>
-      <c r="AA59" s="34" t="s">
-        <v>296</v>
-      </c>
-      <c r="AB59" s="27" t="s">
+      <c r="AD59" s="34" t="s">
         <v>297</v>
       </c>
-      <c r="AC59" s="34" t="s">
-        <v>551</v>
-      </c>
-      <c r="AD59" s="34" t="s">
-        <v>298</v>
-      </c>
       <c r="AE59" s="61" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9638,22 +9631,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
+        <v>551</v>
+      </c>
+      <c r="AC60" s="34" t="s">
         <v>552</v>
-      </c>
-      <c r="AC60" s="34" t="s">
-        <v>553</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9661,22 +9654,22 @@
         <v>126</v>
       </c>
       <c r="B61" s="54" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H61" s="35">
         <v>0.1</v>
@@ -9718,7 +9711,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="V61" s="26">
         <v>60.45333865137971</v>
@@ -9727,28 +9720,28 @@
         <v>22.126007672556039</v>
       </c>
       <c r="X61" s="22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="Y61" s="34" t="s">
+        <v>553</v>
+      </c>
+      <c r="Z61" s="34" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA61" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="AB61" s="46" t="s">
         <v>554</v>
       </c>
-      <c r="Z61" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="AA61" s="34" t="s">
+      <c r="AC61" s="34" t="s">
+        <v>555</v>
+      </c>
+      <c r="AD61" s="34" t="s">
         <v>270</v>
       </c>
-      <c r="AB61" s="46" t="s">
-        <v>555</v>
-      </c>
-      <c r="AC61" s="34" t="s">
-        <v>556</v>
-      </c>
-      <c r="AD61" s="34" t="s">
-        <v>271</v>
-      </c>
       <c r="AE61" s="65" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>
@@ -9836,155 +9829,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="84" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="78" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="73" t="s">
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+    </row>
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="90" t="s">
         <v>315</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-    </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="93" t="s">
+      <c r="B4" s="75"/>
+      <c r="C4" s="83" t="s">
         <v>316</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="82" t="s">
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+    </row>
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="87" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="75"/>
+      <c r="C5" s="83" t="s">
         <v>317</v>
       </c>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-    </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="90" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="82" t="s">
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
+    </row>
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="85" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="75"/>
+      <c r="C6" s="83" t="s">
         <v>318</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-    </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="88" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="82" t="s">
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+    </row>
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="86" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="75"/>
+      <c r="C7" s="83" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-    </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="89" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="77"/>
-      <c r="C7" s="82" t="s">
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+    </row>
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="89" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="75"/>
+      <c r="C8" s="83" t="s">
         <v>320</v>
       </c>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
-    </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="92" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="77"/>
-      <c r="C8" s="82" t="s">
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+    </row>
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="93" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="75"/>
+      <c r="C9" s="83" t="s">
         <v>321</v>
       </c>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-    </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="85" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="77"/>
-      <c r="C9" s="82" t="s">
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="91" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="75"/>
+      <c r="C10" s="83" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="83" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="77"/>
-      <c r="C10" s="82" t="s">
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="78" t="s">
         <v>323</v>
       </c>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="73" t="s">
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+    </row>
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="92" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="74"/>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-    </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="84" t="s">
+      <c r="B13" s="75"/>
+      <c r="C13" s="83" t="s">
         <v>325</v>
       </c>
-      <c r="B13" s="77"/>
-      <c r="C13" s="82" t="s">
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
+    </row>
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="88" t="s">
         <v>326</v>
       </c>
-      <c r="D13" s="74"/>
-      <c r="E13" s="74"/>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="91" t="s">
+      <c r="B14" s="75"/>
+      <c r="C14" s="83" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="77"/>
-      <c r="C14" s="82" t="s">
+      <c r="D14" s="76"/>
+      <c r="E14" s="76"/>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="82" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="74"/>
-      <c r="E14" s="74"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="86" t="s">
+      <c r="B15" s="75"/>
+      <c r="C15" s="83" t="s">
         <v>329</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="82" t="s">
-        <v>330</v>
-      </c>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="42"/>
       <c r="B19" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10001,13 +10001,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10015,26 +10008,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -10275,10 +10248,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10301,20 +10305,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>